<commit_message>
start adding factory_vars. see if modified xls is saved in git
</commit_message>
<xml_diff>
--- a/TestCampaign/ROVCleaver UniversalSetup.xlsx
+++ b/TestCampaign/ROVCleaver UniversalSetup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/TestInputFiles/TestCampaigns/BEK Test UniversalSetup/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/PythonProgs/ROVCleaver_on_Dropbox/TestCampaign/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F377F7A5-22DC-D640-B95E-80695A632667}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7EA7A98-7DF7-FB43-A5AC-A43167471E5C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="24440" windowHeight="11500" activeTab="1" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25940" windowHeight="14100" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="39" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <definedName name="postfix" localSheetId="4">'Load VL checklist group5'!#REF!</definedName>
     <definedName name="postfix" localSheetId="8">'Load VL checklist group4'!#REF!</definedName>
     <definedName name="postfix">'Load VL checklist group5'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Setup!$G$1:$L$189</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Setup!$G$1:$L$192</definedName>
     <definedName name="state" localSheetId="8">'Load VL checklist group4'!$B$2</definedName>
     <definedName name="state">'Load VL checklist group5'!$B$2</definedName>
   </definedNames>
@@ -518,7 +518,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="712">
   <si>
     <t>File</t>
   </si>
@@ -1962,9 +1962,6 @@
   </si>
   <si>
     <t>xl_first_code_sheet</t>
-  </si>
-  <si>
-    <t>False,("splitfield","str")</t>
   </si>
   <si>
     <t>False,("dupe_key_sort_tuples", "pythobj")</t>
@@ -2332,12 +2329,6 @@
     <t>Don't need STATE because it's auto added if files are split by county</t>
   </si>
   <si>
-    <t>SPLIT FIELD</t>
-  </si>
-  <si>
-    <t>Almost always county (used to separate files for Sincere)</t>
-  </si>
-  <si>
     <t>NUMBER OF ROWS TO READ</t>
   </si>
   <si>
@@ -2510,9 +2501,6 @@
   </si>
   <si>
     <t>Automatically prefixed with the state-county, and post-fixed with file counter if addresses are split up because of Sincere maximum count per file</t>
-  </si>
-  <si>
-    <t>Field used to split concatenated file.  Most often County but can be other (eg, District) or a custom group created in modicode code (eg, age group such as "Over 50")</t>
   </si>
   <si>
     <t xml:space="preserve">Allows testing on a small number of records to make sure setup and logic is working.  Value also applies to COMBINED operation, so a low value likely prevents checking of combined data.  Probably use 1001 to check FORMAT files, then up to 999,999 and COMBINE.  Note: Header counts as 1 row so only 1000 addresses are read from each input file when value set set to 1001.  </t>
@@ -2701,6 +2689,33 @@
   </si>
   <si>
     <t xml:space="preserve">  #  Use lagest number in pull_group on FileList?</t>
+  </si>
+  <si>
+    <t>Often blank, used if 'grouping'</t>
+  </si>
+  <si>
+    <t>CAMPAIGN SPLIT VARIABLE(S)</t>
+  </si>
+  <si>
+    <t>FACTORY SPLIT VARIABLE(S)</t>
+  </si>
+  <si>
+    <t>Along with Factory fields, used to split concatenated file.  Most often County but can be other (eg, District) or a custom group created in modicode code (eg, age group such as "Over 50")</t>
+  </si>
+  <si>
+    <t>race,age</t>
+  </si>
+  <si>
+    <t>Used to split at factory level if multiple factories are being loaded with addresses from one combined file.  Most often blank but can be other (eg, District) or a custom group created in modicode code (eg, age group such as "Over 50")</t>
+  </si>
+  <si>
+    <t>False,("splitfield","str",{'str_case':'l'})</t>
+  </si>
+  <si>
+    <t>False,("xl_factory_vars","str",{'str_case':'l'})</t>
+  </si>
+  <si>
+    <t>Almost always county (used to separate files for Sincere along with factory_vars)</t>
   </si>
 </sst>
 </file>
@@ -3131,7 +3146,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
@@ -3280,6 +3295,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="4" builtinId="3"/>
@@ -3603,7 +3619,7 @@
     <tabColor rgb="FFFFFF00"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AD191"/>
+  <dimension ref="A1:AD194"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1" outlineLevel="3"/>
@@ -3635,13 +3651,13 @@
         <v>463</v>
       </c>
       <c r="F1" s="81" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="G1" s="64" t="s">
         <v>289</v>
       </c>
       <c r="J1" s="87" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="K1" s="63"/>
       <c r="L1" s="63"/>
@@ -3664,7 +3680,7 @@
         <v>3</v>
       </c>
       <c r="G3" s="27" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="16" thickBot="1">
@@ -3675,10 +3691,10 @@
         <v>4</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="L4" s="62" t="s">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="M4" s="62"/>
       <c r="N4" s="14"/>
@@ -3700,16 +3716,16 @@
         <v>465</v>
       </c>
       <c r="F5" s="81" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="G5" s="65" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H5" s="66" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="L5" s="62" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
       <c r="M5" s="62"/>
       <c r="N5" s="14"/>
@@ -3722,7 +3738,7 @@
         <v>6</v>
       </c>
       <c r="M6" s="62" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
       <c r="N6" s="62"/>
     </row>
@@ -3734,7 +3750,7 @@
         <v>7</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="17" thickTop="1" thickBot="1">
@@ -3754,13 +3770,13 @@
         <v>466</v>
       </c>
       <c r="F8" s="81" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="G8" s="65" t="s">
         <v>347</v>
       </c>
       <c r="H8" s="66" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="16" thickTop="1">
@@ -3779,12 +3795,12 @@
         <v>10</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="17" thickTop="1" thickBot="1">
       <c r="A11" s="57" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B11">
         <v>62</v>
@@ -3796,16 +3812,16 @@
         <v>1</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F11" s="83" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="G11" s="65" t="s">
+        <v>587</v>
+      </c>
+      <c r="H11" s="66" t="s">
         <v>588</v>
-      </c>
-      <c r="H11" s="66" t="s">
-        <v>589</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="16" thickTop="1">
@@ -3825,12 +3841,12 @@
         <v>13</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="17" thickTop="1" thickBot="1">
       <c r="A14" s="57" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B14">
         <v>105</v>
@@ -3842,16 +3858,16 @@
         <v>1</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F14" s="81" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="G14" s="65" t="s">
         <v>374</v>
       </c>
       <c r="H14" s="66" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="16" thickTop="1">
@@ -3871,10 +3887,10 @@
         <v>16</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" ht="17" thickTop="1" thickBot="1">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="17" thickTop="1" thickBot="1">
       <c r="A17" t="b">
         <v>1</v>
       </c>
@@ -3888,19 +3904,19 @@
         <v>1</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>481</v>
+        <v>709</v>
       </c>
       <c r="F17" s="81" t="s">
-        <v>652</v>
+        <v>706</v>
       </c>
       <c r="G17" s="67" t="s">
         <v>19</v>
       </c>
       <c r="H17" s="66" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" ht="16" thickTop="1">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="16" thickTop="1">
       <c r="B18">
         <v>95</v>
       </c>
@@ -3909,699 +3925,665 @@
       </c>
       <c r="G18" s="43"/>
     </row>
-    <row r="19" spans="1:20" ht="16" thickBot="1">
+    <row r="19" spans="1:14" ht="16" thickBot="1">
       <c r="B19">
+        <v>93</v>
+      </c>
+      <c r="C19">
+        <v>18.2</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="17" thickTop="1" thickBot="1">
+      <c r="A20" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20">
+        <v>94</v>
+      </c>
+      <c r="C20">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="D20" s="92" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>710</v>
+      </c>
+      <c r="F20" s="81" t="s">
+        <v>708</v>
+      </c>
+      <c r="G20" s="67" t="s">
+        <v>707</v>
+      </c>
+      <c r="H20" s="66" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="16" thickTop="1">
+      <c r="C21">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="G21" s="43"/>
+    </row>
+    <row r="22" spans="1:14" ht="16" thickBot="1">
+      <c r="B22">
         <v>18</v>
       </c>
-      <c r="C19">
+      <c r="C22">
         <v>19</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G22" s="1" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="17" thickTop="1" thickBot="1">
+      <c r="A23" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23">
+        <v>19</v>
+      </c>
+      <c r="C23">
+        <v>20</v>
+      </c>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>471</v>
+      </c>
+      <c r="F23" s="83" t="s">
+        <v>649</v>
+      </c>
+      <c r="G23" s="67">
+        <v>1001</v>
+      </c>
+      <c r="H23" s="68" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="16" thickTop="1">
+      <c r="B24">
+        <v>20</v>
+      </c>
+      <c r="C24">
+        <v>21</v>
+      </c>
+      <c r="E24" s="15"/>
+    </row>
+    <row r="25" spans="1:14" ht="16" thickBot="1">
+      <c r="B25">
+        <v>34</v>
+      </c>
+      <c r="C25">
+        <v>22</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="17" thickTop="1" thickBot="1">
+      <c r="A26" s="57" t="s">
+        <v>486</v>
+      </c>
+      <c r="B26">
+        <v>35</v>
+      </c>
+      <c r="C26">
+        <v>23</v>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>506</v>
+      </c>
+      <c r="G26" s="67" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" s="66" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="16" thickTop="1">
+      <c r="B27">
+        <v>36</v>
+      </c>
+      <c r="C27">
+        <v>24</v>
+      </c>
+      <c r="G27" s="4"/>
+    </row>
+    <row r="28" spans="1:14">
+      <c r="B28">
+        <v>10</v>
+      </c>
+      <c r="C28">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="21">
+      <c r="B29">
+        <v>11</v>
+      </c>
+      <c r="C29">
+        <v>26</v>
+      </c>
+      <c r="G29" s="27" t="s">
         <v>594</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="17" thickTop="1" thickBot="1">
-      <c r="A20" t="b">
-        <v>1</v>
-      </c>
-      <c r="B20">
+    <row r="30" spans="1:14" ht="19">
+      <c r="B30">
+        <v>139</v>
+      </c>
+      <c r="C30">
+        <v>27</v>
+      </c>
+      <c r="G30" s="69" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
+      <c r="B31">
+        <v>140</v>
+      </c>
+      <c r="C31">
+        <v>28</v>
+      </c>
+      <c r="F31" s="81" t="s">
+        <v>651</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="H31" s="88" t="s">
+        <v>672</v>
+      </c>
+      <c r="L31" s="62" t="s">
+        <v>691</v>
+      </c>
+      <c r="M31" s="62"/>
+      <c r="N31" s="14"/>
+    </row>
+    <row r="32" spans="1:14" ht="16" thickBot="1">
+      <c r="B32">
+        <v>14</v>
+      </c>
+      <c r="C32">
+        <v>29</v>
+      </c>
+      <c r="G32" s="66" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="A33" t="b">
+        <v>1</v>
+      </c>
+      <c r="B33">
+        <v>141</v>
+      </c>
+      <c r="C33">
+        <v>30</v>
+      </c>
+      <c r="D33" t="b">
+        <v>1</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>468</v>
+      </c>
+      <c r="F33" s="83" t="s">
+        <v>533</v>
+      </c>
+      <c r="G33" s="70" t="s">
+        <v>348</v>
+      </c>
+      <c r="H33" s="70" t="s">
+        <v>201</v>
+      </c>
+      <c r="I33" s="70" t="s">
+        <v>204</v>
+      </c>
+      <c r="J33" s="70" t="s">
+        <v>205</v>
+      </c>
+      <c r="K33" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="L33" s="70" t="s">
+        <v>48</v>
+      </c>
+      <c r="M33" s="70" t="s">
+        <v>207</v>
+      </c>
+      <c r="N33" s="70" t="s">
+        <v>208</v>
+      </c>
+      <c r="O33" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="P33" s="70" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q33" s="71" t="s">
+        <v>211</v>
+      </c>
+      <c r="R33" s="71"/>
+      <c r="S33" s="71"/>
+      <c r="T33" s="71"/>
+    </row>
+    <row r="34" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="A34" t="b">
+        <v>1</v>
+      </c>
+      <c r="B34">
+        <v>142</v>
+      </c>
+      <c r="C34">
+        <v>31</v>
+      </c>
+      <c r="D34" t="b">
+        <v>1</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>469</v>
+      </c>
+      <c r="F34" s="81" t="s">
+        <v>277</v>
+      </c>
+      <c r="G34" s="71" t="s">
+        <v>348</v>
+      </c>
+      <c r="H34" s="71" t="s">
+        <v>20</v>
+      </c>
+      <c r="I34" s="71" t="s">
+        <v>22</v>
+      </c>
+      <c r="J34" s="71" t="s">
+        <v>23</v>
+      </c>
+      <c r="K34" s="71" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="C20">
+      <c r="M34" s="71" t="s">
+        <v>54</v>
+      </c>
+      <c r="N34" s="71" t="s">
+        <v>15</v>
+      </c>
+      <c r="O34" s="71" t="s">
+        <v>16</v>
+      </c>
+      <c r="P34" s="71" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q34" s="71" t="s">
+        <v>21</v>
+      </c>
+      <c r="R34" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="S34" s="71" t="s">
+        <v>378</v>
+      </c>
+      <c r="T34" s="70" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="A35" t="b">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>143</v>
+      </c>
+      <c r="C35">
+        <v>32</v>
+      </c>
+      <c r="D35" t="b">
+        <v>1</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>470</v>
+      </c>
+      <c r="F35" s="83" t="s">
+        <v>650</v>
+      </c>
+      <c r="G35" s="79"/>
+      <c r="H35" s="80"/>
+      <c r="I35" s="80"/>
+      <c r="J35" s="91" t="s">
+        <v>270</v>
+      </c>
+      <c r="K35" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" ht="16" thickTop="1">
+      <c r="B36">
+        <v>149</v>
+      </c>
+      <c r="C36">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" ht="16" thickBot="1">
+      <c r="B37">
+        <v>150</v>
+      </c>
+      <c r="C37">
+        <v>34</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="A38" s="57" t="s">
+        <v>490</v>
+      </c>
+      <c r="B38">
+        <v>151</v>
+      </c>
+      <c r="C38">
+        <v>35</v>
+      </c>
+      <c r="D38" t="b">
+        <v>1</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>519</v>
+      </c>
+      <c r="F38" s="81" t="s">
+        <v>666</v>
+      </c>
+      <c r="G38" s="71" t="s">
+        <v>54</v>
+      </c>
+      <c r="H38" s="66" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" ht="16" thickTop="1">
+      <c r="B39">
+        <v>152</v>
+      </c>
+      <c r="C39">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" ht="16" thickBot="1">
+      <c r="B40">
+        <v>155</v>
+      </c>
+      <c r="C40">
+        <v>37</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="H40" s="66" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="A41" t="b">
+        <v>1</v>
+      </c>
+      <c r="B41">
+        <v>156</v>
+      </c>
+      <c r="C41">
+        <v>38</v>
+      </c>
+      <c r="D41" t="b">
+        <v>1</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>473</v>
+      </c>
+      <c r="F41" s="81" t="s">
+        <v>667</v>
+      </c>
+      <c r="G41" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="D20" t="b">
-        <v>1</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>471</v>
-      </c>
-      <c r="F20" s="83" t="s">
+      <c r="H41" s="71" t="s">
+        <v>22</v>
+      </c>
+      <c r="I41" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="J41" s="71" t="s">
+        <v>16</v>
+      </c>
+      <c r="K41" s="71" t="s">
+        <v>21</v>
+      </c>
+      <c r="L41" s="71" t="s">
+        <v>17</v>
+      </c>
+      <c r="M41" s="71" t="s">
+        <v>24</v>
+      </c>
+      <c r="N41" s="71" t="s">
+        <v>23</v>
+      </c>
+      <c r="O41" s="71" t="s">
+        <v>19</v>
+      </c>
+      <c r="P41" s="71" t="s">
+        <v>364</v>
+      </c>
+      <c r="Q41" s="71" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" ht="16" thickTop="1">
+      <c r="B42">
+        <v>157</v>
+      </c>
+      <c r="C42">
+        <v>39</v>
+      </c>
+      <c r="F42" s="83"/>
+    </row>
+    <row r="43" spans="1:20" ht="16" thickBot="1">
+      <c r="B43">
+        <v>191</v>
+      </c>
+      <c r="C43">
+        <v>40</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="A44" s="57" t="s">
+        <v>492</v>
+      </c>
+      <c r="B44">
+        <v>192</v>
+      </c>
+      <c r="C44">
+        <v>41</v>
+      </c>
+      <c r="D44" t="b">
+        <v>1</v>
+      </c>
+      <c r="E44" s="15" t="s">
+        <v>510</v>
+      </c>
+      <c r="F44" s="81" t="s">
+        <v>279</v>
+      </c>
+      <c r="G44" s="72" t="s">
+        <v>348</v>
+      </c>
+      <c r="H44" s="66" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" ht="16" thickTop="1">
+      <c r="B45">
+        <v>193</v>
+      </c>
+      <c r="C45">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20" ht="16" thickBot="1">
+      <c r="B46">
+        <v>194</v>
+      </c>
+      <c r="C46">
+        <v>43</v>
+      </c>
+      <c r="G46" t="s">
+        <v>604</v>
+      </c>
+      <c r="H46" s="66"/>
+    </row>
+    <row r="47" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="A47" s="57" t="s">
+        <v>493</v>
+      </c>
+      <c r="B47">
+        <v>195</v>
+      </c>
+      <c r="C47">
+        <v>44</v>
+      </c>
+      <c r="D47" t="b">
+        <v>1</v>
+      </c>
+      <c r="E47" s="15" t="s">
+        <v>511</v>
+      </c>
+      <c r="F47" s="81" t="s">
+        <v>278</v>
+      </c>
+      <c r="G47" s="72" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" ht="16" thickTop="1">
+      <c r="B48">
+        <v>196</v>
+      </c>
+      <c r="C48">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" ht="16" thickBot="1">
+      <c r="B49">
+        <v>187</v>
+      </c>
+      <c r="C49">
+        <v>46</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A50" s="57" t="s">
+        <v>491</v>
+      </c>
+      <c r="B50">
+        <v>188</v>
+      </c>
+      <c r="C50">
+        <v>47</v>
+      </c>
+      <c r="D50" t="b">
+        <v>1</v>
+      </c>
+      <c r="E50" s="15" t="s">
+        <v>509</v>
+      </c>
+      <c r="F50" s="81" t="s">
+        <v>652</v>
+      </c>
+      <c r="G50" s="73" t="b">
+        <v>0</v>
+      </c>
+      <c r="H50" s="66" t="s">
         <v>653</v>
       </c>
-      <c r="G20" s="67">
-        <v>1001</v>
-      </c>
-      <c r="H20" s="68" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" ht="16" thickTop="1">
-      <c r="B21">
-        <v>20</v>
-      </c>
-      <c r="C21">
-        <v>21</v>
-      </c>
-      <c r="E21" s="15"/>
-    </row>
-    <row r="22" spans="1:20" ht="16" thickBot="1">
-      <c r="B22">
-        <v>34</v>
-      </c>
-      <c r="C22">
-        <v>22</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" ht="17" thickTop="1" thickBot="1">
-      <c r="A23" s="57" t="s">
-        <v>487</v>
-      </c>
-      <c r="B23">
-        <v>35</v>
-      </c>
-      <c r="C23">
-        <v>23</v>
-      </c>
-      <c r="D23" t="b">
-        <v>1</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>507</v>
-      </c>
-      <c r="G23" s="67" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="66" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" ht="16" thickTop="1">
-      <c r="B24">
-        <v>36</v>
-      </c>
-      <c r="C24">
-        <v>24</v>
-      </c>
-      <c r="G24" s="4"/>
-    </row>
-    <row r="25" spans="1:20">
-      <c r="B25">
-        <v>10</v>
-      </c>
-      <c r="C25">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" ht="21">
-      <c r="B26">
-        <v>11</v>
-      </c>
-      <c r="C26">
-        <v>26</v>
-      </c>
-      <c r="G26" s="27" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" ht="19">
-      <c r="B27">
-        <v>139</v>
-      </c>
-      <c r="C27">
-        <v>27</v>
-      </c>
-      <c r="G27" s="69" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20">
-      <c r="B28">
-        <v>140</v>
-      </c>
-      <c r="C28">
-        <v>28</v>
-      </c>
-      <c r="F28" s="81" t="s">
-        <v>655</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>599</v>
-      </c>
-      <c r="H28" s="88" t="s">
-        <v>676</v>
-      </c>
-      <c r="L28" s="62" t="s">
-        <v>695</v>
-      </c>
-      <c r="M28" s="62"/>
-      <c r="N28" s="14"/>
-    </row>
-    <row r="29" spans="1:20" ht="16" thickBot="1">
-      <c r="B29">
-        <v>14</v>
-      </c>
-      <c r="C29">
-        <v>29</v>
-      </c>
-      <c r="G29" s="66" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" ht="17" thickTop="1" thickBot="1">
-      <c r="A30" t="b">
-        <v>1</v>
-      </c>
-      <c r="B30">
-        <v>141</v>
-      </c>
-      <c r="C30">
-        <v>30</v>
-      </c>
-      <c r="D30" t="b">
-        <v>1</v>
-      </c>
-      <c r="E30" s="15" t="s">
-        <v>468</v>
-      </c>
-      <c r="F30" s="83" t="s">
-        <v>534</v>
-      </c>
-      <c r="G30" s="70" t="s">
-        <v>348</v>
-      </c>
-      <c r="H30" s="70" t="s">
-        <v>201</v>
-      </c>
-      <c r="I30" s="70" t="s">
-        <v>204</v>
-      </c>
-      <c r="J30" s="70" t="s">
-        <v>205</v>
-      </c>
-      <c r="K30" s="70" t="s">
-        <v>206</v>
-      </c>
-      <c r="L30" s="70" t="s">
+    </row>
+    <row r="51" spans="1:16" ht="16" thickTop="1">
+      <c r="B51">
+        <v>189</v>
+      </c>
+      <c r="C51">
         <v>48</v>
       </c>
-      <c r="M30" s="70" t="s">
-        <v>207</v>
-      </c>
-      <c r="N30" s="70" t="s">
-        <v>208</v>
-      </c>
-      <c r="O30" s="70" t="s">
-        <v>209</v>
-      </c>
-      <c r="P30" s="70" t="s">
-        <v>210</v>
-      </c>
-      <c r="Q30" s="71" t="s">
-        <v>211</v>
-      </c>
-      <c r="R30" s="71"/>
-      <c r="S30" s="71"/>
-      <c r="T30" s="71"/>
-    </row>
-    <row r="31" spans="1:20" ht="17" thickTop="1" thickBot="1">
-      <c r="A31" t="b">
-        <v>1</v>
-      </c>
-      <c r="B31">
-        <v>142</v>
-      </c>
-      <c r="C31">
-        <v>31</v>
-      </c>
-      <c r="D31" t="b">
-        <v>1</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>469</v>
-      </c>
-      <c r="F31" s="81" t="s">
-        <v>277</v>
-      </c>
-      <c r="G31" s="71" t="s">
-        <v>348</v>
-      </c>
-      <c r="H31" s="71" t="s">
-        <v>20</v>
-      </c>
-      <c r="I31" s="71" t="s">
-        <v>22</v>
-      </c>
-      <c r="J31" s="71" t="s">
-        <v>23</v>
-      </c>
-      <c r="K31" s="71" t="s">
-        <v>24</v>
-      </c>
-      <c r="L31" s="71" t="s">
-        <v>19</v>
-      </c>
-      <c r="M31" s="71" t="s">
-        <v>54</v>
-      </c>
-      <c r="N31" s="71" t="s">
-        <v>15</v>
-      </c>
-      <c r="O31" s="71" t="s">
-        <v>16</v>
-      </c>
-      <c r="P31" s="71" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q31" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="R31" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="S31" s="71" t="s">
-        <v>378</v>
-      </c>
-      <c r="T31" s="70" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" ht="17" thickTop="1" thickBot="1">
-      <c r="A32" t="b">
-        <v>1</v>
-      </c>
-      <c r="B32">
-        <v>143</v>
-      </c>
-      <c r="C32">
-        <v>32</v>
-      </c>
-      <c r="D32" t="b">
-        <v>1</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>470</v>
-      </c>
-      <c r="F32" s="83" t="s">
-        <v>654</v>
-      </c>
-      <c r="G32" s="79"/>
-      <c r="H32" s="80"/>
-      <c r="I32" s="80"/>
-      <c r="J32" s="91" t="s">
-        <v>270</v>
-      </c>
-      <c r="K32" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" ht="16" thickTop="1">
-      <c r="B33">
-        <v>149</v>
-      </c>
-      <c r="C33">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" ht="16" thickBot="1">
-      <c r="B34">
-        <v>150</v>
-      </c>
-      <c r="C34">
-        <v>34</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" ht="17" thickTop="1" thickBot="1">
-      <c r="A35" s="57" t="s">
-        <v>491</v>
-      </c>
-      <c r="B35">
-        <v>151</v>
-      </c>
-      <c r="C35">
-        <v>35</v>
-      </c>
-      <c r="D35" t="b">
-        <v>1</v>
-      </c>
-      <c r="E35" s="15" t="s">
-        <v>520</v>
-      </c>
-      <c r="F35" s="81" t="s">
-        <v>670</v>
-      </c>
-      <c r="G35" s="71" t="s">
-        <v>54</v>
-      </c>
-      <c r="H35" s="66" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" ht="16" thickTop="1">
-      <c r="B36">
-        <v>152</v>
-      </c>
-      <c r="C36">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" ht="16" thickBot="1">
-      <c r="B37">
-        <v>155</v>
-      </c>
-      <c r="C37">
-        <v>37</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>603</v>
-      </c>
-      <c r="H37" s="66" t="s">
-        <v>604</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" ht="17" thickTop="1" thickBot="1">
-      <c r="A38" t="b">
-        <v>1</v>
-      </c>
-      <c r="B38">
-        <v>156</v>
-      </c>
-      <c r="C38">
-        <v>38</v>
-      </c>
-      <c r="D38" t="b">
-        <v>1</v>
-      </c>
-      <c r="E38" s="15" t="s">
-        <v>473</v>
-      </c>
-      <c r="F38" s="81" t="s">
-        <v>671</v>
-      </c>
-      <c r="G38" s="71" t="s">
-        <v>20</v>
-      </c>
-      <c r="H38" s="71" t="s">
-        <v>22</v>
-      </c>
-      <c r="I38" s="71" t="s">
-        <v>14</v>
-      </c>
-      <c r="J38" s="71" t="s">
-        <v>16</v>
-      </c>
-      <c r="K38" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="L38" s="71" t="s">
-        <v>17</v>
-      </c>
-      <c r="M38" s="71" t="s">
-        <v>24</v>
-      </c>
-      <c r="N38" s="71" t="s">
-        <v>23</v>
-      </c>
-      <c r="O38" s="71" t="s">
-        <v>19</v>
-      </c>
-      <c r="P38" s="71" t="s">
-        <v>364</v>
-      </c>
-      <c r="Q38" s="71" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" ht="16" thickTop="1">
-      <c r="B39">
-        <v>157</v>
-      </c>
-      <c r="C39">
-        <v>39</v>
-      </c>
-      <c r="F39" s="83"/>
-    </row>
-    <row r="40" spans="1:17" ht="16" thickBot="1">
-      <c r="B40">
-        <v>191</v>
-      </c>
-      <c r="C40">
-        <v>40</v>
-      </c>
-      <c r="G40" s="1" t="s">
+    </row>
+    <row r="52" spans="1:16" ht="19">
+      <c r="B52">
+        <v>97</v>
+      </c>
+      <c r="C52">
+        <v>49</v>
+      </c>
+      <c r="G52" s="69" t="s">
         <v>605</v>
       </c>
-    </row>
-    <row r="41" spans="1:17" ht="17" thickTop="1" thickBot="1">
-      <c r="A41" s="57" t="s">
-        <v>493</v>
-      </c>
-      <c r="B41">
-        <v>192</v>
-      </c>
-      <c r="C41">
-        <v>41</v>
-      </c>
-      <c r="D41" t="b">
-        <v>1</v>
-      </c>
-      <c r="E41" s="15" t="s">
-        <v>511</v>
-      </c>
-      <c r="F41" s="81" t="s">
-        <v>279</v>
-      </c>
-      <c r="G41" s="72" t="s">
-        <v>348</v>
-      </c>
-      <c r="H41" s="66" t="s">
+      <c r="H52" s="66" t="s">
         <v>606</v>
       </c>
     </row>
-    <row r="42" spans="1:17" ht="16" thickTop="1">
-      <c r="B42">
-        <v>193</v>
-      </c>
-      <c r="C42">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" spans="1:17" ht="16" thickBot="1">
-      <c r="B43">
-        <v>194</v>
-      </c>
-      <c r="C43">
-        <v>43</v>
-      </c>
-      <c r="G43" t="s">
+    <row r="53" spans="1:16" ht="49" thickBot="1">
+      <c r="B53" s="78">
+        <v>97.5</v>
+      </c>
+      <c r="C53">
+        <v>50</v>
+      </c>
+      <c r="G53" s="4" t="s">
         <v>607</v>
       </c>
-      <c r="H43" s="66"/>
-    </row>
-    <row r="44" spans="1:17" ht="17" thickTop="1" thickBot="1">
-      <c r="A44" s="57" t="s">
-        <v>494</v>
-      </c>
-      <c r="B44">
-        <v>195</v>
-      </c>
-      <c r="C44">
-        <v>44</v>
-      </c>
-      <c r="D44" t="b">
-        <v>1</v>
-      </c>
-      <c r="E44" s="15" t="s">
-        <v>512</v>
-      </c>
-      <c r="F44" s="81" t="s">
-        <v>278</v>
-      </c>
-      <c r="G44" s="72" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="45" spans="1:17" ht="16" thickTop="1">
-      <c r="B45">
-        <v>196</v>
-      </c>
-      <c r="C45">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="46" spans="1:17" ht="16" thickBot="1">
-      <c r="B46">
-        <v>187</v>
-      </c>
-      <c r="C46">
-        <v>46</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" ht="17" thickTop="1" thickBot="1">
-      <c r="A47" s="57" t="s">
-        <v>492</v>
-      </c>
-      <c r="B47">
-        <v>188</v>
-      </c>
-      <c r="C47">
-        <v>47</v>
-      </c>
-      <c r="D47" t="b">
-        <v>1</v>
-      </c>
-      <c r="E47" s="15" t="s">
-        <v>510</v>
-      </c>
-      <c r="F47" s="81" t="s">
-        <v>656</v>
-      </c>
-      <c r="G47" s="73" t="b">
+      <c r="H53" s="35" t="s">
+        <v>608</v>
+      </c>
+      <c r="I53" s="35" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A54" s="60" t="b">
+        <v>1</v>
+      </c>
+      <c r="B54">
+        <v>98</v>
+      </c>
+      <c r="C54">
+        <v>51</v>
+      </c>
+      <c r="D54" s="60" t="b">
+        <v>1</v>
+      </c>
+      <c r="E54" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="F54" s="81" t="s">
+        <v>535</v>
+      </c>
+      <c r="G54" s="72" t="s">
+        <v>387</v>
+      </c>
+      <c r="H54" s="74" t="b">
         <v>0</v>
-      </c>
-      <c r="H47" s="66" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="48" spans="1:17" ht="16" thickTop="1">
-      <c r="B48">
-        <v>189</v>
-      </c>
-      <c r="C48">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" ht="19">
-      <c r="B49">
-        <v>97</v>
-      </c>
-      <c r="C49">
-        <v>49</v>
-      </c>
-      <c r="G49" s="69" t="s">
-        <v>608</v>
-      </c>
-      <c r="H49" s="66" t="s">
-        <v>609</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" ht="49" thickBot="1">
-      <c r="B50" s="78">
-        <v>97.5</v>
-      </c>
-      <c r="C50">
-        <v>50</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>610</v>
-      </c>
-      <c r="H50" s="35" t="s">
-        <v>611</v>
-      </c>
-      <c r="I50" s="35" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A51" s="60" t="b">
-        <v>1</v>
-      </c>
-      <c r="B51">
-        <v>98</v>
-      </c>
-      <c r="C51">
-        <v>51</v>
-      </c>
-      <c r="D51" s="60" t="b">
-        <v>1</v>
-      </c>
-      <c r="E51" s="15" t="s">
-        <v>526</v>
-      </c>
-      <c r="F51" s="81" t="s">
-        <v>536</v>
-      </c>
-      <c r="G51" s="72" t="s">
-        <v>387</v>
-      </c>
-      <c r="H51" s="74" t="b">
-        <v>0</v>
-      </c>
-      <c r="I51" s="72" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A52" t="b">
-        <v>1</v>
-      </c>
-      <c r="B52">
-        <v>99</v>
-      </c>
-      <c r="C52">
-        <v>52</v>
-      </c>
-      <c r="D52" t="b">
-        <v>1</v>
-      </c>
-      <c r="E52" s="15" t="s">
-        <v>527</v>
-      </c>
-      <c r="F52" s="83"/>
-      <c r="G52" s="72"/>
-      <c r="H52" s="72" t="b">
-        <v>0</v>
-      </c>
-      <c r="I52" s="72" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A53" t="b">
-        <v>1</v>
-      </c>
-      <c r="B53">
-        <v>100</v>
-      </c>
-      <c r="C53">
-        <v>53</v>
-      </c>
-      <c r="D53" t="b">
-        <v>1</v>
-      </c>
-      <c r="E53" s="15" t="s">
-        <v>528</v>
-      </c>
-      <c r="G53" s="72" t="s">
-        <v>455</v>
-      </c>
-      <c r="H53" s="72" t="b">
-        <v>0</v>
-      </c>
-      <c r="I53" s="72" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A54" t="b">
-        <v>1</v>
-      </c>
-      <c r="B54">
-        <v>101</v>
-      </c>
-      <c r="C54">
-        <v>54</v>
-      </c>
-      <c r="D54" t="b">
-        <v>1</v>
-      </c>
-      <c r="E54" s="15" t="s">
-        <v>529</v>
-      </c>
-      <c r="G54" s="72" t="s">
-        <v>390</v>
-      </c>
-      <c r="H54" s="72" t="b">
-        <v>1</v>
       </c>
       <c r="I54" s="72" t="b">
         <v>1</v>
@@ -4612,1508 +4594,1585 @@
         <v>1</v>
       </c>
       <c r="B55">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C55">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D55" t="b">
         <v>1</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>530</v>
-      </c>
-      <c r="G55" s="72" t="s">
-        <v>545</v>
-      </c>
+        <v>526</v>
+      </c>
+      <c r="F55" s="83"/>
+      <c r="G55" s="72"/>
       <c r="H55" s="72" t="b">
         <v>0</v>
       </c>
       <c r="I55" s="72" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" ht="16" thickTop="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A56" t="b">
+        <v>1</v>
+      </c>
       <c r="B56">
+        <v>100</v>
+      </c>
+      <c r="C56">
+        <v>53</v>
+      </c>
+      <c r="D56" t="b">
+        <v>1</v>
+      </c>
+      <c r="E56" s="15" t="s">
+        <v>527</v>
+      </c>
+      <c r="G56" s="72" t="s">
+        <v>455</v>
+      </c>
+      <c r="H56" s="72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I56" s="72" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A57" t="b">
+        <v>1</v>
+      </c>
+      <c r="B57">
+        <v>101</v>
+      </c>
+      <c r="C57">
+        <v>54</v>
+      </c>
+      <c r="D57" t="b">
+        <v>1</v>
+      </c>
+      <c r="E57" s="15" t="s">
+        <v>528</v>
+      </c>
+      <c r="G57" s="72" t="s">
+        <v>390</v>
+      </c>
+      <c r="H57" s="72" t="b">
+        <v>1</v>
+      </c>
+      <c r="I57" s="72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A58" t="b">
+        <v>1</v>
+      </c>
+      <c r="B58">
+        <v>102</v>
+      </c>
+      <c r="C58">
+        <v>55</v>
+      </c>
+      <c r="D58" t="b">
+        <v>1</v>
+      </c>
+      <c r="E58" s="15" t="s">
+        <v>529</v>
+      </c>
+      <c r="G58" s="72" t="s">
+        <v>544</v>
+      </c>
+      <c r="H58" s="72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" s="72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" ht="16" thickTop="1">
+      <c r="B59">
         <v>102.5</v>
       </c>
-      <c r="C56">
+      <c r="C59">
         <v>56</v>
       </c>
-      <c r="E56" s="15"/>
-    </row>
-    <row r="57" spans="1:16">
-      <c r="B57">
+      <c r="E59" s="15"/>
+    </row>
+    <row r="60" spans="1:16">
+      <c r="B60">
         <v>103</v>
       </c>
-      <c r="C57">
+      <c r="C60">
         <v>57</v>
       </c>
     </row>
-    <row r="58" spans="1:16" ht="19">
-      <c r="B58">
+    <row r="61" spans="1:16" ht="19">
+      <c r="B61">
         <v>16</v>
       </c>
-      <c r="C58">
+      <c r="C61">
         <v>58</v>
       </c>
-      <c r="G58" s="69" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" ht="16" thickBot="1">
-      <c r="B59">
-        <v>12</v>
-      </c>
-      <c r="C59">
-        <v>59</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>613</v>
-      </c>
-      <c r="L59" s="62" t="s">
-        <v>660</v>
-      </c>
-      <c r="M59" s="61"/>
-      <c r="N59" s="61"/>
-      <c r="O59" s="61"/>
-      <c r="P59" s="61"/>
-    </row>
-    <row r="60" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A60" t="b">
-        <v>1</v>
-      </c>
-      <c r="B60">
-        <v>13</v>
-      </c>
-      <c r="C60">
-        <v>60</v>
-      </c>
-      <c r="D60" t="b">
-        <v>1</v>
-      </c>
-      <c r="E60" t="s">
-        <v>472</v>
-      </c>
-      <c r="F60" s="81" t="s">
-        <v>659</v>
-      </c>
-      <c r="G60" s="72" t="s">
-        <v>276</v>
-      </c>
-      <c r="H60" s="66" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="61" spans="1:16" ht="16" thickTop="1">
-      <c r="B61">
-        <v>15</v>
-      </c>
-      <c r="C61">
-        <v>61</v>
+      <c r="G61" s="69" t="s">
+        <v>611</v>
       </c>
     </row>
     <row r="62" spans="1:16" ht="16" thickBot="1">
       <c r="B62">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C62">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>615</v>
-      </c>
+        <v>610</v>
+      </c>
+      <c r="L62" s="62" t="s">
+        <v>656</v>
+      </c>
+      <c r="M62" s="61"/>
+      <c r="N62" s="61"/>
+      <c r="O62" s="61"/>
+      <c r="P62" s="61"/>
     </row>
     <row r="63" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A63" s="57" t="s">
-        <v>485</v>
+      <c r="A63" t="b">
+        <v>1</v>
       </c>
       <c r="B63">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C63">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D63" t="b">
         <v>1</v>
       </c>
-      <c r="E63" s="15" t="s">
-        <v>506</v>
+      <c r="E63" t="s">
+        <v>472</v>
       </c>
       <c r="F63" s="81" t="s">
-        <v>532</v>
-      </c>
-      <c r="G63" s="73">
-        <v>3</v>
+        <v>655</v>
+      </c>
+      <c r="G63" s="72" t="s">
+        <v>276</v>
       </c>
       <c r="H63" s="66" t="s">
-        <v>616</v>
+        <v>654</v>
       </c>
     </row>
     <row r="64" spans="1:16" ht="16" thickTop="1">
       <c r="B64">
+        <v>15</v>
+      </c>
+      <c r="C64">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" ht="16" thickBot="1">
+      <c r="B65">
+        <v>23</v>
+      </c>
+      <c r="C65">
+        <v>62</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" ht="17" thickTop="1" thickBot="1">
+      <c r="A66" s="57" t="s">
+        <v>484</v>
+      </c>
+      <c r="B66">
+        <v>24</v>
+      </c>
+      <c r="C66">
+        <v>63</v>
+      </c>
+      <c r="D66" t="b">
+        <v>1</v>
+      </c>
+      <c r="E66" s="15" t="s">
+        <v>505</v>
+      </c>
+      <c r="F66" s="81" t="s">
+        <v>531</v>
+      </c>
+      <c r="G66" s="73">
+        <v>3</v>
+      </c>
+      <c r="H66" s="66" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" ht="16" thickTop="1">
+      <c r="B67">
         <v>25</v>
       </c>
-      <c r="C64">
+      <c r="C67">
         <v>64</v>
       </c>
     </row>
-    <row r="65" spans="1:15">
-      <c r="B65">
+    <row r="68" spans="1:15">
+      <c r="B68">
         <v>37</v>
       </c>
-      <c r="C65">
+      <c r="C68">
         <v>65</v>
       </c>
-      <c r="G65" s="1" t="s">
-        <v>662</v>
-      </c>
-      <c r="H65" s="66" t="s">
-        <v>663</v>
-      </c>
-      <c r="L65" s="62" t="s">
-        <v>617</v>
-      </c>
-      <c r="M65" s="61"/>
-      <c r="N65" s="61"/>
-      <c r="O65" s="61"/>
-    </row>
-    <row r="66" spans="1:15">
-      <c r="A66" t="b">
-        <v>1</v>
-      </c>
-      <c r="B66">
-        <v>38</v>
-      </c>
-      <c r="C66">
-        <v>66</v>
-      </c>
-      <c r="D66" t="b">
-        <v>1</v>
-      </c>
-      <c r="E66" s="15" t="s">
-        <v>537</v>
-      </c>
-      <c r="F66" s="81" t="s">
-        <v>661</v>
-      </c>
-      <c r="G66" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="67" spans="1:15">
-      <c r="B67">
-        <v>39</v>
-      </c>
-      <c r="C67">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" ht="16" thickBot="1">
-      <c r="B68">
-        <v>41</v>
-      </c>
-      <c r="C68">
-        <v>68</v>
-      </c>
-      <c r="G68" s="32" t="s">
-        <v>664</v>
-      </c>
-      <c r="H68" s="84" t="s">
-        <v>665</v>
-      </c>
-      <c r="I68" s="14"/>
-      <c r="J68" s="79"/>
-      <c r="K68" s="79"/>
+      <c r="G68" s="1" t="s">
+        <v>658</v>
+      </c>
+      <c r="H68" s="66" t="s">
+        <v>659</v>
+      </c>
       <c r="L68" s="62" t="s">
-        <v>673</v>
+        <v>614</v>
       </c>
       <c r="M68" s="61"/>
       <c r="N68" s="61"/>
       <c r="O68" s="61"/>
     </row>
-    <row r="69" spans="1:15" ht="17" thickTop="1" thickBot="1">
+    <row r="69" spans="1:15">
       <c r="A69" t="b">
         <v>1</v>
       </c>
       <c r="B69">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C69">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D69" t="b">
         <v>1</v>
       </c>
       <c r="E69" s="15" t="s">
-        <v>482</v>
+        <v>536</v>
       </c>
       <c r="F69" s="81" t="s">
-        <v>543</v>
-      </c>
-      <c r="G69" s="72" t="s">
-        <v>483</v>
-      </c>
-      <c r="L69" s="62" t="s">
-        <v>617</v>
-      </c>
-      <c r="M69" s="61"/>
-      <c r="N69" s="61"/>
-    </row>
-    <row r="70" spans="1:15" ht="16" thickTop="1">
+        <v>657</v>
+      </c>
+      <c r="G69" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15">
       <c r="B70">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C70">
-        <v>70</v>
-      </c>
-      <c r="G70" s="26"/>
+        <v>67</v>
+      </c>
     </row>
     <row r="71" spans="1:15" ht="16" thickBot="1">
       <c r="B71">
-        <v>199</v>
+        <v>41</v>
       </c>
       <c r="C71">
-        <v>71</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>618</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="G71" s="32" t="s">
+        <v>660</v>
+      </c>
+      <c r="H71" s="84" t="s">
+        <v>661</v>
+      </c>
+      <c r="I71" s="14"/>
+      <c r="J71" s="79"/>
+      <c r="K71" s="79"/>
+      <c r="L71" s="62" t="s">
+        <v>669</v>
+      </c>
+      <c r="M71" s="61"/>
+      <c r="N71" s="61"/>
+      <c r="O71" s="61"/>
     </row>
     <row r="72" spans="1:15" ht="17" thickTop="1" thickBot="1">
-      <c r="A72" s="57" t="s">
-        <v>495</v>
+      <c r="A72" t="b">
+        <v>1</v>
       </c>
       <c r="B72">
-        <v>200</v>
+        <v>42</v>
       </c>
       <c r="C72">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D72" t="b">
         <v>1</v>
       </c>
       <c r="E72" s="15" t="s">
-        <v>513</v>
+        <v>481</v>
       </c>
       <c r="F72" s="81" t="s">
-        <v>672</v>
-      </c>
-      <c r="G72" s="73" t="b">
-        <v>1</v>
-      </c>
-      <c r="H72" s="66" t="s">
-        <v>619</v>
-      </c>
+        <v>542</v>
+      </c>
+      <c r="G72" s="72" t="s">
+        <v>482</v>
+      </c>
+      <c r="L72" s="62" t="s">
+        <v>614</v>
+      </c>
+      <c r="M72" s="61"/>
+      <c r="N72" s="61"/>
     </row>
     <row r="73" spans="1:15" ht="16" thickTop="1">
       <c r="B73">
-        <v>201</v>
+        <v>43</v>
       </c>
       <c r="C73">
-        <v>73</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="G73" s="26"/>
     </row>
     <row r="74" spans="1:15" ht="16" thickBot="1">
       <c r="B74">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="C74">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>620</v>
-      </c>
-      <c r="L74" s="62" t="s">
-        <v>621</v>
-      </c>
-      <c r="M74" s="62"/>
-      <c r="N74" s="14"/>
+        <v>615</v>
+      </c>
     </row>
     <row r="75" spans="1:15" ht="17" thickTop="1" thickBot="1">
       <c r="A75" s="57" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="B75">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="C75">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D75" t="b">
         <v>1</v>
       </c>
       <c r="E75" s="15" t="s">
-        <v>514</v>
-      </c>
-      <c r="F75" s="85" t="s">
-        <v>535</v>
+        <v>512</v>
+      </c>
+      <c r="F75" s="81" t="s">
+        <v>668</v>
       </c>
       <c r="G75" s="73" t="b">
         <v>1</v>
       </c>
       <c r="H75" s="66" t="s">
-        <v>622</v>
+        <v>616</v>
       </c>
     </row>
     <row r="76" spans="1:15" ht="16" thickTop="1">
       <c r="B76">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="C76">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="77" spans="1:15" ht="16" thickBot="1">
       <c r="B77">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C77">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>623</v>
-      </c>
+        <v>617</v>
+      </c>
+      <c r="L77" s="62" t="s">
+        <v>618</v>
+      </c>
+      <c r="M77" s="62"/>
+      <c r="N77" s="14"/>
     </row>
     <row r="78" spans="1:15" ht="17" thickTop="1" thickBot="1">
-      <c r="A78" t="s">
-        <v>497</v>
+      <c r="A78" s="57" t="s">
+        <v>495</v>
       </c>
       <c r="B78">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C78">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D78" t="b">
         <v>1</v>
       </c>
       <c r="E78" s="15" t="s">
-        <v>522</v>
-      </c>
-      <c r="F78" s="81" t="s">
-        <v>666</v>
-      </c>
-      <c r="G78" s="73" t="s">
-        <v>196</v>
+        <v>513</v>
+      </c>
+      <c r="F78" s="85" t="s">
+        <v>534</v>
+      </c>
+      <c r="G78" s="73" t="b">
+        <v>1</v>
       </c>
       <c r="H78" s="66" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
     </row>
     <row r="79" spans="1:15" ht="16" thickTop="1">
       <c r="B79">
+        <v>212</v>
+      </c>
+      <c r="C79">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" ht="16" thickBot="1">
+      <c r="B80">
+        <v>214</v>
+      </c>
+      <c r="C80">
+        <v>77</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="81" spans="1:30" ht="17" thickTop="1" thickBot="1">
+      <c r="A81" t="s">
+        <v>496</v>
+      </c>
+      <c r="B81">
+        <v>215</v>
+      </c>
+      <c r="C81">
+        <v>78</v>
+      </c>
+      <c r="D81" t="b">
+        <v>1</v>
+      </c>
+      <c r="E81" s="15" t="s">
+        <v>521</v>
+      </c>
+      <c r="F81" s="81" t="s">
+        <v>662</v>
+      </c>
+      <c r="G81" s="73" t="s">
+        <v>196</v>
+      </c>
+      <c r="H81" s="66" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="82" spans="1:30" ht="16" thickTop="1">
+      <c r="B82">
         <v>216</v>
       </c>
-      <c r="C79">
+      <c r="C82">
         <v>79</v>
       </c>
     </row>
-    <row r="80" spans="1:15">
-      <c r="B80">
+    <row r="83" spans="1:30">
+      <c r="B83">
         <v>17</v>
       </c>
-      <c r="C80">
+      <c r="C83">
         <v>80</v>
       </c>
     </row>
-    <row r="81" spans="1:30" ht="19">
-      <c r="B81">
+    <row r="84" spans="1:30" ht="19">
+      <c r="B84">
         <v>21</v>
       </c>
-      <c r="C81">
+      <c r="C84">
         <v>81</v>
       </c>
-      <c r="G81" s="69" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="82" spans="1:30" ht="16" thickBot="1">
-      <c r="B82">
-        <v>247</v>
-      </c>
-      <c r="C82">
-        <v>82</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>626</v>
-      </c>
-    </row>
-    <row r="83" spans="1:30" ht="17" thickTop="1" thickBot="1">
-      <c r="A83" s="57" t="s">
-        <v>500</v>
-      </c>
-      <c r="B83">
-        <v>248</v>
-      </c>
-      <c r="C83">
-        <v>83</v>
-      </c>
-      <c r="D83" t="b">
-        <v>1</v>
-      </c>
-      <c r="E83" s="15" t="s">
-        <v>515</v>
-      </c>
-      <c r="F83" s="81" t="s">
-        <v>667</v>
-      </c>
-      <c r="G83" s="73" t="b">
-        <v>1</v>
-      </c>
-      <c r="H83" s="66" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="84" spans="1:30" ht="16" thickTop="1">
-      <c r="B84">
-        <v>249</v>
-      </c>
-      <c r="C84">
-        <v>84</v>
-      </c>
-      <c r="G84" s="4"/>
+      <c r="G84" s="69" t="s">
+        <v>622</v>
+      </c>
     </row>
     <row r="85" spans="1:30" ht="16" thickBot="1">
       <c r="B85">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C85">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
     </row>
     <row r="86" spans="1:30" ht="17" thickTop="1" thickBot="1">
       <c r="A86" s="57" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B86">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C86">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D86" t="b">
         <v>1</v>
       </c>
       <c r="E86" s="15" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="F86" s="81" t="s">
-        <v>668</v>
+        <v>663</v>
       </c>
       <c r="G86" s="73" t="b">
         <v>1</v>
       </c>
       <c r="H86" s="66" t="s">
-        <v>629</v>
+        <v>624</v>
       </c>
     </row>
     <row r="87" spans="1:30" ht="16" thickTop="1">
       <c r="B87">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C87">
-        <v>87</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="G87" s="4"/>
     </row>
     <row r="88" spans="1:30" ht="16" thickBot="1">
       <c r="B88">
-        <v>28</v>
+        <v>252</v>
       </c>
       <c r="C88">
-        <v>88</v>
-      </c>
-      <c r="G88" s="86" t="s">
-        <v>329</v>
-      </c>
-      <c r="N88" s="62" t="s">
-        <v>630</v>
-      </c>
-      <c r="O88" s="61"/>
-      <c r="P88" s="61"/>
-      <c r="Q88" s="61"/>
-      <c r="AD88" s="28"/>
+        <v>85</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>625</v>
+      </c>
     </row>
     <row r="89" spans="1:30" ht="17" thickTop="1" thickBot="1">
       <c r="A89" s="57" t="s">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="B89">
-        <v>29</v>
+        <v>253</v>
       </c>
       <c r="C89">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D89" t="b">
         <v>1</v>
       </c>
       <c r="E89" s="15" t="s">
-        <v>518</v>
-      </c>
-      <c r="F89" s="85" t="s">
-        <v>533</v>
-      </c>
-      <c r="G89" s="75">
-        <v>3</v>
+        <v>515</v>
+      </c>
+      <c r="F89" s="81" t="s">
+        <v>664</v>
+      </c>
+      <c r="G89" s="73" t="b">
+        <v>1</v>
       </c>
       <c r="H89" s="66" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
     </row>
     <row r="90" spans="1:30" ht="16" thickTop="1">
       <c r="B90">
+        <v>254</v>
+      </c>
+      <c r="C90">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="91" spans="1:30" ht="16" thickBot="1">
+      <c r="B91">
+        <v>28</v>
+      </c>
+      <c r="C91">
+        <v>88</v>
+      </c>
+      <c r="G91" s="86" t="s">
+        <v>329</v>
+      </c>
+      <c r="N91" s="62" t="s">
+        <v>627</v>
+      </c>
+      <c r="O91" s="61"/>
+      <c r="P91" s="61"/>
+      <c r="Q91" s="61"/>
+      <c r="AD91" s="28"/>
+    </row>
+    <row r="92" spans="1:30" ht="17" thickTop="1" thickBot="1">
+      <c r="A92" s="57" t="s">
+        <v>485</v>
+      </c>
+      <c r="B92">
+        <v>29</v>
+      </c>
+      <c r="C92">
+        <v>89</v>
+      </c>
+      <c r="D92" t="b">
+        <v>1</v>
+      </c>
+      <c r="E92" s="15" t="s">
+        <v>517</v>
+      </c>
+      <c r="F92" s="85" t="s">
+        <v>532</v>
+      </c>
+      <c r="G92" s="75">
+        <v>3</v>
+      </c>
+      <c r="H92" s="66" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="93" spans="1:30" ht="16" thickTop="1">
+      <c r="B93">
         <v>30</v>
       </c>
-      <c r="C90">
+      <c r="C93">
         <v>90</v>
       </c>
-      <c r="G90" s="76" t="s">
+      <c r="G93" s="76" t="s">
         <v>266</v>
       </c>
-      <c r="L90" s="62" t="s">
-        <v>632</v>
-      </c>
-      <c r="M90" s="61"/>
-      <c r="N90" s="61"/>
-    </row>
-    <row r="91" spans="1:30">
-      <c r="B91">
+      <c r="L93" s="62" t="s">
+        <v>629</v>
+      </c>
+      <c r="M93" s="61"/>
+      <c r="N93" s="61"/>
+    </row>
+    <row r="94" spans="1:30">
+      <c r="B94">
         <v>22</v>
       </c>
-      <c r="C91">
+      <c r="C94">
         <v>91</v>
       </c>
     </row>
-    <row r="92" spans="1:30" ht="16" thickBot="1">
-      <c r="B92">
+    <row r="95" spans="1:30" ht="16" thickBot="1">
+      <c r="B95">
         <v>109</v>
       </c>
-      <c r="C92">
+      <c r="C95">
         <v>92</v>
       </c>
-      <c r="G92" s="1" t="s">
-        <v>633</v>
-      </c>
-      <c r="I92" s="17"/>
-    </row>
-    <row r="93" spans="1:30" ht="17" thickTop="1" thickBot="1">
-      <c r="A93" s="57" t="s">
-        <v>490</v>
-      </c>
-      <c r="B93">
+      <c r="G95" s="1" t="s">
+        <v>630</v>
+      </c>
+      <c r="I95" s="17"/>
+    </row>
+    <row r="96" spans="1:30" ht="17" thickTop="1" thickBot="1">
+      <c r="A96" s="57" t="s">
+        <v>489</v>
+      </c>
+      <c r="B96">
         <v>110</v>
       </c>
-      <c r="C93">
+      <c r="C96">
         <v>93</v>
       </c>
-      <c r="D93" t="b">
-        <v>1</v>
-      </c>
-      <c r="E93" s="15" t="s">
-        <v>519</v>
-      </c>
-      <c r="F93" s="81" t="s">
-        <v>674</v>
-      </c>
-      <c r="G93" s="75">
+      <c r="D96" t="b">
+        <v>1</v>
+      </c>
+      <c r="E96" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="F96" s="81" t="s">
+        <v>670</v>
+      </c>
+      <c r="G96" s="75">
         <v>25000</v>
       </c>
-      <c r="H93" s="66" t="s">
-        <v>634</v>
-      </c>
-      <c r="J93" s="76"/>
-      <c r="K93" s="76"/>
-    </row>
-    <row r="94" spans="1:30" ht="16" thickTop="1">
-      <c r="B94">
+      <c r="H96" s="66" t="s">
+        <v>631</v>
+      </c>
+      <c r="J96" s="76"/>
+      <c r="K96" s="76"/>
+    </row>
+    <row r="97" spans="1:16" ht="16" thickTop="1">
+      <c r="B97">
         <v>111</v>
       </c>
-      <c r="C94">
+      <c r="C97">
         <v>94</v>
       </c>
     </row>
-    <row r="95" spans="1:30">
-      <c r="B95">
+    <row r="98" spans="1:16">
+      <c r="B98">
         <v>26</v>
       </c>
-      <c r="C95">
+      <c r="C98">
         <v>95</v>
       </c>
     </row>
-    <row r="96" spans="1:30" ht="21">
-      <c r="B96">
+    <row r="99" spans="1:16" ht="21">
+      <c r="B99">
         <v>27</v>
       </c>
-      <c r="C96">
+      <c r="C99">
         <v>96</v>
       </c>
-      <c r="G96" s="27" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="97" spans="1:16" ht="16" thickBot="1">
-      <c r="B97">
-        <v>219</v>
-      </c>
-      <c r="C97">
-        <v>97</v>
-      </c>
-      <c r="G97" s="1" t="s">
-        <v>635</v>
-      </c>
-      <c r="H97" s="89" t="s">
-        <v>678</v>
-      </c>
-      <c r="I97" s="79"/>
-    </row>
-    <row r="98" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A98" t="s">
-        <v>474</v>
-      </c>
-      <c r="B98">
-        <v>220</v>
-      </c>
-      <c r="C98">
-        <v>98</v>
-      </c>
-      <c r="D98" t="b">
-        <v>1</v>
-      </c>
-      <c r="E98" s="15" t="s">
-        <v>475</v>
-      </c>
-      <c r="F98" s="81" t="s">
-        <v>677</v>
-      </c>
-      <c r="G98" s="73" t="b">
-        <v>1</v>
-      </c>
-      <c r="H98" s="66" t="s">
-        <v>596</v>
-      </c>
-      <c r="L98" s="62" t="s">
-        <v>645</v>
-      </c>
-      <c r="M98" s="62"/>
-      <c r="N98" s="62"/>
-    </row>
-    <row r="99" spans="1:16" ht="16" thickTop="1">
-      <c r="B99">
-        <v>221</v>
-      </c>
-      <c r="C99">
-        <v>99</v>
-      </c>
-      <c r="H99" s="66"/>
+      <c r="G99" s="27" t="s">
+        <v>641</v>
+      </c>
     </row>
     <row r="100" spans="1:16" ht="16" thickBot="1">
       <c r="B100">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C100">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G100" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="H100" s="66" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="101" spans="1:16" s="81" customFormat="1" ht="17" thickTop="1" thickBot="1">
-      <c r="A101" s="81" t="s">
-        <v>480</v>
-      </c>
-      <c r="B101" s="81">
-        <v>224</v>
+        <v>632</v>
+      </c>
+      <c r="H100" s="89" t="s">
+        <v>674</v>
+      </c>
+      <c r="I100" s="79"/>
+    </row>
+    <row r="101" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A101" t="s">
+        <v>474</v>
+      </c>
+      <c r="B101">
+        <v>220</v>
       </c>
       <c r="C101">
-        <v>101</v>
-      </c>
-      <c r="D101" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="E101" s="83" t="s">
-        <v>523</v>
-      </c>
-      <c r="F101" s="90" t="s">
-        <v>679</v>
-      </c>
-      <c r="G101" s="72" t="s">
-        <v>284</v>
+        <v>98</v>
+      </c>
+      <c r="D101" t="b">
+        <v>1</v>
+      </c>
+      <c r="E101" s="15" t="s">
+        <v>475</v>
+      </c>
+      <c r="F101" s="81" t="s">
+        <v>673</v>
+      </c>
+      <c r="G101" s="73" t="b">
+        <v>1</v>
       </c>
       <c r="H101" s="66" t="s">
-        <v>638</v>
+        <v>593</v>
       </c>
       <c r="L101" s="62" t="s">
-        <v>691</v>
+        <v>642</v>
       </c>
       <c r="M101" s="62"/>
       <c r="N101" s="62"/>
-      <c r="O101" s="62"/>
-      <c r="P101" s="62"/>
     </row>
     <row r="102" spans="1:16" ht="16" thickTop="1">
       <c r="B102">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C102">
-        <v>102</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="H102" s="66"/>
     </row>
     <row r="103" spans="1:16" ht="16" thickBot="1">
       <c r="B103">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="C103">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G103" s="1" t="s">
-        <v>639</v>
+        <v>633</v>
       </c>
       <c r="H103" s="66" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="104" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A104" t="s">
-        <v>477</v>
-      </c>
-      <c r="B104">
-        <v>229</v>
+        <v>634</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" s="81" customFormat="1" ht="17" thickTop="1" thickBot="1">
+      <c r="A104" s="81" t="s">
+        <v>480</v>
+      </c>
+      <c r="B104" s="81">
+        <v>224</v>
       </c>
       <c r="C104">
-        <v>104</v>
-      </c>
-      <c r="D104" t="b">
-        <v>1</v>
-      </c>
-      <c r="E104" s="15" t="s">
-        <v>476</v>
+        <v>101</v>
+      </c>
+      <c r="D104" s="81" t="b">
+        <v>1</v>
+      </c>
+      <c r="E104" s="83" t="s">
+        <v>522</v>
       </c>
       <c r="F104" s="90" t="s">
-        <v>680</v>
-      </c>
-      <c r="G104" s="73" t="b">
-        <v>1</v>
+        <v>675</v>
+      </c>
+      <c r="G104" s="72" t="s">
+        <v>284</v>
       </c>
       <c r="H104" s="66" t="s">
-        <v>640</v>
-      </c>
+        <v>635</v>
+      </c>
+      <c r="L104" s="62" t="s">
+        <v>687</v>
+      </c>
+      <c r="M104" s="62"/>
+      <c r="N104" s="62"/>
+      <c r="O104" s="62"/>
+      <c r="P104" s="62"/>
     </row>
     <row r="105" spans="1:16" ht="16" thickTop="1">
       <c r="B105">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="C105">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="106" spans="1:16" ht="16" thickBot="1">
       <c r="B106">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C106">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G106" s="1" t="s">
-        <v>641</v>
+        <v>636</v>
+      </c>
+      <c r="H106" s="66" t="s">
+        <v>677</v>
       </c>
     </row>
     <row r="107" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A107" s="57" t="s">
-        <v>498</v>
+      <c r="A107" t="s">
+        <v>477</v>
       </c>
       <c r="B107">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C107">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D107" t="b">
         <v>1</v>
       </c>
       <c r="E107" s="15" t="s">
-        <v>524</v>
+        <v>476</v>
       </c>
       <c r="F107" s="90" t="s">
-        <v>687</v>
-      </c>
-      <c r="G107" s="72" t="s">
-        <v>285</v>
+        <v>676</v>
+      </c>
+      <c r="G107" s="73" t="b">
+        <v>1</v>
       </c>
       <c r="H107" s="66" t="s">
-        <v>638</v>
-      </c>
-      <c r="L107" s="62" t="s">
-        <v>682</v>
-      </c>
-      <c r="M107" s="62"/>
-      <c r="N107" s="62"/>
-      <c r="O107" s="62"/>
-      <c r="P107" s="62"/>
+        <v>637</v>
+      </c>
     </row>
     <row r="108" spans="1:16" ht="16" thickTop="1">
       <c r="B108">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="C108">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="109" spans="1:16" ht="16" thickBot="1">
       <c r="B109">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C109">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G109" s="1" t="s">
-        <v>642</v>
-      </c>
-      <c r="H109" s="66" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="110" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A110" s="57" t="s">
+        <v>497</v>
+      </c>
+      <c r="B110">
+        <v>233</v>
+      </c>
+      <c r="C110">
+        <v>107</v>
+      </c>
+      <c r="D110" t="b">
+        <v>1</v>
+      </c>
+      <c r="E110" s="15" t="s">
+        <v>523</v>
+      </c>
+      <c r="F110" s="90" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="110" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A110" t="s">
-        <v>478</v>
-      </c>
-      <c r="B110">
-        <v>238</v>
-      </c>
-      <c r="C110">
-        <v>110</v>
-      </c>
-      <c r="D110" t="b">
-        <v>1</v>
-      </c>
-      <c r="E110" s="15" t="s">
-        <v>479</v>
-      </c>
-      <c r="F110" s="90" t="s">
-        <v>684</v>
-      </c>
-      <c r="G110" s="73" t="b">
-        <v>1</v>
+      <c r="G110" s="72" t="s">
+        <v>285</v>
       </c>
       <c r="H110" s="66" t="s">
-        <v>640</v>
-      </c>
+        <v>635</v>
+      </c>
+      <c r="L110" s="62" t="s">
+        <v>678</v>
+      </c>
+      <c r="M110" s="62"/>
+      <c r="N110" s="62"/>
+      <c r="O110" s="62"/>
+      <c r="P110" s="62"/>
     </row>
     <row r="111" spans="1:16" ht="16" thickTop="1">
       <c r="B111">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="C111">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="112" spans="1:16" ht="16" thickBot="1">
       <c r="B112">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C112">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="G112" s="1" t="s">
-        <v>643</v>
+        <v>639</v>
+      </c>
+      <c r="H112" s="66" t="s">
+        <v>679</v>
       </c>
     </row>
     <row r="113" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A113" s="57" t="s">
-        <v>499</v>
+      <c r="A113" t="s">
+        <v>478</v>
       </c>
       <c r="B113">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="C113">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D113" t="b">
         <v>1</v>
       </c>
       <c r="E113" s="15" t="s">
-        <v>525</v>
+        <v>479</v>
       </c>
       <c r="F113" s="90" t="s">
-        <v>685</v>
-      </c>
-      <c r="G113" s="72" t="s">
-        <v>286</v>
+        <v>680</v>
+      </c>
+      <c r="G113" s="73" t="b">
+        <v>1</v>
       </c>
       <c r="H113" s="66" t="s">
-        <v>638</v>
-      </c>
-      <c r="L113" s="62" t="s">
-        <v>686</v>
-      </c>
-      <c r="M113" s="62"/>
-      <c r="N113" s="62"/>
-      <c r="O113" s="62"/>
-      <c r="P113" s="62"/>
+        <v>637</v>
+      </c>
     </row>
     <row r="114" spans="1:16" ht="16" thickTop="1">
       <c r="B114">
+        <v>239</v>
+      </c>
+      <c r="C114">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" ht="16" thickBot="1">
+      <c r="B115">
+        <v>241</v>
+      </c>
+      <c r="C115">
+        <v>112</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A116" s="57" t="s">
+        <v>498</v>
+      </c>
+      <c r="B116">
+        <v>242</v>
+      </c>
+      <c r="C116">
+        <v>113</v>
+      </c>
+      <c r="D116" t="b">
+        <v>1</v>
+      </c>
+      <c r="E116" s="15" t="s">
+        <v>524</v>
+      </c>
+      <c r="F116" s="90" t="s">
+        <v>681</v>
+      </c>
+      <c r="G116" s="72" t="s">
+        <v>286</v>
+      </c>
+      <c r="H116" s="66" t="s">
+        <v>635</v>
+      </c>
+      <c r="L116" s="62" t="s">
+        <v>682</v>
+      </c>
+      <c r="M116" s="62"/>
+      <c r="N116" s="62"/>
+      <c r="O116" s="62"/>
+      <c r="P116" s="62"/>
+    </row>
+    <row r="117" spans="1:16" ht="16" thickTop="1">
+      <c r="B117">
         <v>243</v>
       </c>
-      <c r="C114">
+      <c r="C117">
         <v>114</v>
       </c>
     </row>
-    <row r="115" spans="1:16">
-      <c r="B115">
+    <row r="118" spans="1:16">
+      <c r="B118">
         <v>244</v>
       </c>
-      <c r="C115">
+      <c r="C118">
         <v>115</v>
       </c>
     </row>
-    <row r="116" spans="1:16" ht="21">
-      <c r="B116">
+    <row r="119" spans="1:16" ht="21">
+      <c r="B119">
         <v>287</v>
       </c>
-      <c r="C116">
+      <c r="C119">
         <v>116</v>
       </c>
-      <c r="G116" s="27" t="s">
+      <c r="G119" s="27" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="117" spans="1:16" ht="16" thickBot="1">
-      <c r="B117">
-        <v>288</v>
-      </c>
-      <c r="C117">
-        <v>117</v>
-      </c>
-      <c r="G117" t="s">
-        <v>688</v>
-      </c>
-    </row>
-    <row r="118" spans="1:16" ht="17" thickTop="1" thickBot="1">
-      <c r="A118" s="57" t="s">
-        <v>502</v>
-      </c>
-      <c r="B118">
-        <v>289</v>
-      </c>
-      <c r="C118">
-        <v>118</v>
-      </c>
-      <c r="D118" t="b">
-        <v>1</v>
-      </c>
-      <c r="E118" s="15" t="s">
-        <v>517</v>
-      </c>
-      <c r="F118" s="90" t="s">
-        <v>690</v>
-      </c>
-      <c r="G118" s="73" t="b">
-        <v>0</v>
-      </c>
-      <c r="H118" s="66" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="119" spans="1:16" ht="16" thickTop="1">
-      <c r="B119">
-        <v>290</v>
-      </c>
-      <c r="C119">
-        <v>119</v>
-      </c>
-      <c r="G119" s="76"/>
     </row>
     <row r="120" spans="1:16" ht="16" thickBot="1">
       <c r="B120">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="C120">
-        <v>120</v>
-      </c>
-      <c r="G120" s="86" t="s">
-        <v>192</v>
+        <v>117</v>
+      </c>
+      <c r="G120" t="s">
+        <v>684</v>
       </c>
     </row>
     <row r="121" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A121" s="57" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B121">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C121">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D121" t="b">
         <v>1</v>
       </c>
       <c r="E121" s="15" t="s">
-        <v>538</v>
-      </c>
-      <c r="F121" s="85" t="s">
-        <v>540</v>
-      </c>
-      <c r="G121" s="71" t="s">
-        <v>193</v>
+        <v>516</v>
+      </c>
+      <c r="F121" s="90" t="s">
+        <v>686</v>
+      </c>
+      <c r="G121" s="73" t="b">
+        <v>0</v>
+      </c>
+      <c r="H121" s="66" t="s">
+        <v>685</v>
       </c>
     </row>
     <row r="122" spans="1:16" ht="16" thickTop="1">
       <c r="B122">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="C122">
-        <v>122</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="G122" s="76"/>
     </row>
     <row r="123" spans="1:16" ht="16" thickBot="1">
       <c r="B123">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="C123">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G123" s="86" t="s">
-        <v>669</v>
-      </c>
-      <c r="N123" s="77" t="s">
-        <v>646</v>
-      </c>
-      <c r="O123" s="61"/>
-      <c r="P123" s="61"/>
+        <v>192</v>
+      </c>
     </row>
     <row r="124" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A124" s="57" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="B124">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="C124">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D124" t="b">
         <v>1</v>
       </c>
       <c r="E124" s="15" t="s">
+        <v>537</v>
+      </c>
+      <c r="F124" s="85" t="s">
         <v>539</v>
       </c>
-      <c r="F124" s="85" t="s">
-        <v>541</v>
-      </c>
       <c r="G124" s="71" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="125" spans="1:16" ht="16" thickTop="1">
       <c r="B125">
+        <v>295</v>
+      </c>
+      <c r="C125">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="126" spans="1:16" ht="16" thickBot="1">
+      <c r="B126">
+        <v>298</v>
+      </c>
+      <c r="C126">
+        <v>123</v>
+      </c>
+      <c r="G126" s="86" t="s">
+        <v>665</v>
+      </c>
+      <c r="N126" s="77" t="s">
+        <v>643</v>
+      </c>
+      <c r="O126" s="61"/>
+      <c r="P126" s="61"/>
+    </row>
+    <row r="127" spans="1:16" ht="17" thickTop="1" thickBot="1">
+      <c r="A127" s="57" t="s">
+        <v>503</v>
+      </c>
+      <c r="B127">
+        <v>299</v>
+      </c>
+      <c r="C127">
+        <v>124</v>
+      </c>
+      <c r="D127" t="b">
+        <v>1</v>
+      </c>
+      <c r="E127" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="F127" s="85" t="s">
+        <v>540</v>
+      </c>
+      <c r="G127" s="71" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="128" spans="1:16" ht="16" thickTop="1">
+      <c r="B128">
         <v>300</v>
       </c>
-      <c r="C125">
+      <c r="C128">
         <v>125</v>
       </c>
     </row>
-    <row r="126" spans="1:16">
-      <c r="B126">
+    <row r="129" spans="1:14">
+      <c r="B129">
         <v>303</v>
       </c>
-      <c r="C126">
+      <c r="C129">
         <v>126</v>
       </c>
-      <c r="G126" s="21" t="s">
+      <c r="G129" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="H126" s="42" t="s">
+      <c r="H129" s="42" t="s">
         <v>190</v>
       </c>
-      <c r="I126" s="9"/>
-      <c r="J126" s="9"/>
-      <c r="K126" s="9"/>
-      <c r="L126" s="9"/>
-      <c r="N126" s="62" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="127" spans="1:16">
-      <c r="A127" s="57" t="s">
-        <v>505</v>
-      </c>
-      <c r="B127">
+      <c r="I129" s="9"/>
+      <c r="J129" s="9"/>
+      <c r="K129" s="9"/>
+      <c r="L129" s="9"/>
+      <c r="N129" s="62" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="130" spans="1:14">
+      <c r="A130" s="57" t="s">
+        <v>504</v>
+      </c>
+      <c r="B130">
         <v>304</v>
       </c>
-      <c r="C127">
+      <c r="C130">
         <v>127</v>
       </c>
-      <c r="D127" t="b">
-        <v>1</v>
-      </c>
-      <c r="E127" s="15" t="s">
-        <v>521</v>
-      </c>
-      <c r="F127" s="81" t="s">
+      <c r="D130" t="b">
+        <v>1</v>
+      </c>
+      <c r="E130" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="F130" s="81" t="s">
         <v>280</v>
       </c>
-      <c r="G127" t="s">
+      <c r="G130" t="s">
         <v>57</v>
       </c>
-      <c r="H127" t="s">
+      <c r="H130" t="s">
         <v>14</v>
       </c>
-      <c r="I127" t="s">
+      <c r="I130" t="s">
         <v>15</v>
       </c>
-      <c r="J127" t="s">
+      <c r="J130" t="s">
         <v>16</v>
       </c>
-      <c r="N127" s="62" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="130" spans="2:7">
-      <c r="G130" s="14" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="131" spans="2:7">
-      <c r="B131">
+      <c r="N130" s="62" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="133" spans="1:14">
+      <c r="G133" s="14" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="134" spans="1:14">
+      <c r="B134">
         <v>31</v>
       </c>
     </row>
-    <row r="132" spans="2:7">
-      <c r="B132">
+    <row r="135" spans="1:14">
+      <c r="B135">
         <v>32</v>
       </c>
     </row>
-    <row r="133" spans="2:7">
-      <c r="B133">
+    <row r="136" spans="1:14">
+      <c r="B136">
         <v>33</v>
       </c>
-      <c r="G133" s="5" t="s">
+      <c r="G136" s="5" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="134" spans="2:7">
-      <c r="B134">
+    <row r="137" spans="1:14">
+      <c r="B137">
         <v>40</v>
       </c>
-      <c r="G134" s="26"/>
-    </row>
-    <row r="135" spans="2:7">
-      <c r="B135">
+      <c r="G137" s="26"/>
+    </row>
+    <row r="138" spans="1:14">
+      <c r="B138">
         <v>44</v>
       </c>
     </row>
-    <row r="136" spans="2:7">
-      <c r="B136">
+    <row r="139" spans="1:14">
+      <c r="B139">
         <v>58</v>
       </c>
-      <c r="G136" s="4"/>
-    </row>
-    <row r="137" spans="2:7">
-      <c r="B137">
+      <c r="G139" s="4"/>
+    </row>
+    <row r="140" spans="1:14">
+      <c r="B140">
         <v>59</v>
       </c>
     </row>
-    <row r="138" spans="2:7" collapsed="1">
-      <c r="B138">
+    <row r="141" spans="1:14" collapsed="1">
+      <c r="B141">
         <v>60</v>
       </c>
-      <c r="G138" s="5" t="s">
+      <c r="G141" s="5" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="139" spans="2:7">
-      <c r="B139">
+    <row r="142" spans="1:14">
+      <c r="B142">
         <v>64</v>
       </c>
     </row>
-    <row r="140" spans="2:7">
-      <c r="B140">
+    <row r="143" spans="1:14">
+      <c r="B143">
         <v>91</v>
       </c>
-      <c r="G140" s="4"/>
-    </row>
-    <row r="141" spans="2:7">
-      <c r="B141">
+      <c r="G143" s="4"/>
+    </row>
+    <row r="144" spans="1:14">
+      <c r="B144">
         <v>92</v>
       </c>
-      <c r="G141" s="5" t="s">
+      <c r="G144" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="142" spans="2:7">
-      <c r="B142">
+    <row r="145" spans="2:2">
+      <c r="B145">
         <v>96</v>
       </c>
     </row>
-    <row r="143" spans="2:7">
-      <c r="B143">
+    <row r="146" spans="2:2">
+      <c r="B146">
         <v>107</v>
       </c>
     </row>
-    <row r="144" spans="2:7">
-      <c r="B144">
+    <row r="147" spans="2:2">
+      <c r="B147">
         <v>108</v>
       </c>
     </row>
-    <row r="145" spans="2:7">
-      <c r="B145">
+    <row r="148" spans="2:2">
+      <c r="B148">
         <v>112</v>
       </c>
     </row>
-    <row r="146" spans="2:7">
-      <c r="B146">
+    <row r="149" spans="2:2">
+      <c r="B149">
         <v>137</v>
       </c>
     </row>
-    <row r="147" spans="2:7">
-      <c r="B147">
+    <row r="150" spans="2:2">
+      <c r="B150">
         <v>138</v>
       </c>
     </row>
-    <row r="148" spans="2:7">
-      <c r="B148">
+    <row r="151" spans="2:2">
+      <c r="B151">
         <v>144</v>
       </c>
     </row>
-    <row r="149" spans="2:7">
-      <c r="B149">
+    <row r="152" spans="2:2">
+      <c r="B152">
         <v>145</v>
       </c>
     </row>
-    <row r="150" spans="2:7">
-      <c r="B150">
+    <row r="153" spans="2:2">
+      <c r="B153">
         <v>146</v>
       </c>
     </row>
-    <row r="151" spans="2:7">
-      <c r="B151">
+    <row r="154" spans="2:2">
+      <c r="B154">
         <v>147</v>
       </c>
     </row>
-    <row r="152" spans="2:7">
-      <c r="B152">
+    <row r="155" spans="2:2">
+      <c r="B155">
         <v>148</v>
       </c>
     </row>
-    <row r="153" spans="2:7">
-      <c r="B153">
+    <row r="156" spans="2:2">
+      <c r="B156">
         <v>153</v>
       </c>
     </row>
-    <row r="154" spans="2:7">
-      <c r="B154">
+    <row r="157" spans="2:2">
+      <c r="B157">
         <v>154</v>
       </c>
     </row>
-    <row r="155" spans="2:7">
-      <c r="B155">
+    <row r="158" spans="2:2">
+      <c r="B158">
         <v>158</v>
       </c>
     </row>
-    <row r="156" spans="2:7">
-      <c r="B156">
+    <row r="159" spans="2:2">
+      <c r="B159">
         <v>184</v>
       </c>
     </row>
-    <row r="157" spans="2:7">
-      <c r="B157">
+    <row r="160" spans="2:2">
+      <c r="B160">
         <v>185</v>
-      </c>
-    </row>
-    <row r="158" spans="2:7">
-      <c r="B158">
-        <v>186</v>
-      </c>
-      <c r="G158" s="5" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="159" spans="2:7">
-      <c r="B159">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="160" spans="2:7">
-      <c r="B160">
-        <v>197</v>
       </c>
     </row>
     <row r="161" spans="2:7">
       <c r="B161">
-        <v>198</v>
+        <v>186</v>
+      </c>
+      <c r="G161" s="5" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="162" spans="2:7">
       <c r="B162">
-        <v>202</v>
+        <v>190</v>
       </c>
     </row>
     <row r="163" spans="2:7">
       <c r="B163">
-        <v>203</v>
-      </c>
-      <c r="G163" s="4"/>
+        <v>197</v>
+      </c>
     </row>
     <row r="164" spans="2:7">
       <c r="B164">
-        <v>208</v>
+        <v>198</v>
       </c>
     </row>
     <row r="165" spans="2:7">
       <c r="B165">
-        <v>209</v>
-      </c>
-      <c r="G165" s="4"/>
+        <v>202</v>
+      </c>
     </row>
     <row r="166" spans="2:7">
       <c r="B166">
-        <v>213</v>
-      </c>
+        <v>203</v>
+      </c>
+      <c r="G166" s="4"/>
     </row>
     <row r="167" spans="2:7">
       <c r="B167">
-        <v>217</v>
-      </c>
-      <c r="G167" s="4"/>
+        <v>208</v>
+      </c>
     </row>
     <row r="168" spans="2:7">
       <c r="B168">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="G168" s="4"/>
     </row>
     <row r="169" spans="2:7">
       <c r="B169">
-        <v>222</v>
+        <v>213</v>
       </c>
     </row>
     <row r="170" spans="2:7">
       <c r="B170">
-        <v>226</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="G170" s="4"/>
     </row>
     <row r="171" spans="2:7">
       <c r="B171">
-        <v>227</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="G171" s="4"/>
     </row>
     <row r="172" spans="2:7">
       <c r="B172">
-        <v>231</v>
+        <v>222</v>
       </c>
     </row>
     <row r="173" spans="2:7">
       <c r="B173">
-        <v>235</v>
+        <v>226</v>
       </c>
     </row>
     <row r="174" spans="2:7">
       <c r="B174">
-        <v>236</v>
+        <v>227</v>
       </c>
     </row>
     <row r="175" spans="2:7">
       <c r="B175">
-        <v>240</v>
+        <v>231</v>
       </c>
     </row>
     <row r="176" spans="2:7">
       <c r="B176">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="177" spans="2:7">
+      <c r="B177">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="178" spans="2:7">
+      <c r="B178">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="179" spans="2:7">
+      <c r="B179">
         <v>245</v>
       </c>
     </row>
-    <row r="177" spans="2:19">
-      <c r="B177">
+    <row r="180" spans="2:7">
+      <c r="B180">
         <v>246</v>
       </c>
     </row>
-    <row r="178" spans="2:19">
-      <c r="B178">
+    <row r="181" spans="2:7">
+      <c r="B181">
         <v>250</v>
       </c>
     </row>
-    <row r="179" spans="2:19">
-      <c r="B179">
+    <row r="182" spans="2:7">
+      <c r="B182">
         <v>251</v>
       </c>
     </row>
-    <row r="180" spans="2:19">
-      <c r="B180">
+    <row r="183" spans="2:7">
+      <c r="B183">
         <v>255</v>
       </c>
-      <c r="G180" s="1"/>
-    </row>
-    <row r="181" spans="2:19">
-      <c r="B181">
+      <c r="G183" s="1"/>
+    </row>
+    <row r="184" spans="2:7">
+      <c r="B184">
         <v>286</v>
       </c>
     </row>
-    <row r="182" spans="2:19">
-      <c r="B182">
+    <row r="185" spans="2:7">
+      <c r="B185">
         <v>291</v>
       </c>
     </row>
-    <row r="183" spans="2:19">
-      <c r="B183">
+    <row r="186" spans="2:7">
+      <c r="B186">
         <v>292</v>
       </c>
     </row>
-    <row r="184" spans="2:19">
-      <c r="B184">
+    <row r="187" spans="2:7">
+      <c r="B187">
         <v>296</v>
       </c>
     </row>
-    <row r="185" spans="2:19">
-      <c r="B185">
+    <row r="188" spans="2:7">
+      <c r="B188">
         <v>297</v>
       </c>
     </row>
-    <row r="186" spans="2:19">
-      <c r="B186">
+    <row r="189" spans="2:7">
+      <c r="B189">
         <v>301</v>
       </c>
     </row>
-    <row r="187" spans="2:19">
-      <c r="B187">
+    <row r="190" spans="2:7">
+      <c r="B190">
         <v>302</v>
       </c>
     </row>
-    <row r="188" spans="2:19">
-      <c r="B188">
+    <row r="191" spans="2:7">
+      <c r="B191">
         <v>305</v>
       </c>
     </row>
-    <row r="189" spans="2:19">
-      <c r="B189">
+    <row r="192" spans="2:7">
+      <c r="B192">
         <v>306</v>
       </c>
     </row>
-    <row r="190" spans="2:19">
-      <c r="B190">
+    <row r="193" spans="2:19">
+      <c r="B193">
         <v>307</v>
       </c>
     </row>
-    <row r="191" spans="2:19">
-      <c r="B191">
+    <row r="194" spans="2:19">
+      <c r="B194">
         <v>308</v>
       </c>
-      <c r="M191" s="1"/>
-      <c r="N191" s="1"/>
-      <c r="O191" s="1"/>
-      <c r="P191" s="1"/>
-      <c r="Q191" s="1"/>
-      <c r="R191" s="1"/>
-      <c r="S191" s="1"/>
+      <c r="M194" s="1"/>
+      <c r="N194" s="1"/>
+      <c r="O194" s="1"/>
+      <c r="P194" s="1"/>
+      <c r="Q194" s="1"/>
+      <c r="R194" s="1"/>
+      <c r="S194" s="1"/>
     </row>
   </sheetData>
-  <sortState ref="A2:T181">
-    <sortCondition ref="C2:C181"/>
+  <sortState ref="A2:T184">
+    <sortCondition ref="C2:C184"/>
   </sortState>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="76" fitToHeight="9" orientation="portrait" r:id="rId1"/>
@@ -8997,13 +9056,13 @@
         <v>383</v>
       </c>
       <c r="G1" s="51" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H1" s="52" t="s">
         <v>4</v>
       </c>
       <c r="J1" s="53" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="K1" s="14"/>
       <c r="L1" s="14"/>
@@ -9011,19 +9070,16 @@
     </row>
     <row r="2" spans="1:13" ht="15">
       <c r="A2" t="s">
-        <v>562</v>
-      </c>
-      <c r="F2" s="4">
-        <v>5</v>
+        <v>561</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H2" t="s">
         <v>389</v>
       </c>
       <c r="J2" s="53" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="K2" s="14"/>
       <c r="L2" s="14"/>
@@ -9031,19 +9087,19 @@
     </row>
     <row r="3" spans="1:13" ht="15">
       <c r="A3" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F3" s="4">
         <v>4</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="H3" t="s">
         <v>389</v>
       </c>
       <c r="J3" s="53" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="K3" s="14"/>
       <c r="L3" s="14"/>
@@ -9051,19 +9107,19 @@
     </row>
     <row r="4" spans="1:13" ht="15">
       <c r="A4" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F4" s="4">
         <v>3</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="H4" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="J4" s="53" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="K4" s="14"/>
       <c r="L4" s="14"/>
@@ -9083,7 +9139,7 @@
         <v>2</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="H5" t="s">
         <v>389</v>
@@ -9100,13 +9156,13 @@
         <v>1</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="H6" t="s">
         <v>389</v>
       </c>
       <c r="J6" s="53" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="K6" s="14"/>
       <c r="L6" s="14"/>
@@ -9114,13 +9170,13 @@
     </row>
     <row r="7" spans="1:13" ht="15">
       <c r="A7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="F7" s="4">
         <v>5</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H7" t="s">
         <v>389</v>
@@ -9140,7 +9196,7 @@
         <v>4</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="H8" t="s">
         <v>389</v>
@@ -9148,97 +9204,97 @@
     </row>
     <row r="9" spans="1:13" ht="15">
       <c r="A9" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F9" s="4">
         <v>3</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H9" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15">
       <c r="A10" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="F10" s="4">
         <v>2</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="H10" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="15">
       <c r="A11" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="F11" s="4">
         <v>1</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="H11" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15">
       <c r="A12" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="F12" s="4">
         <v>5</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="H12" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15">
       <c r="A13" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="F13" s="4">
         <v>4</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="H13" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15">
       <c r="A14" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="F14" s="4">
         <v>3</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H14" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15">
       <c r="A15" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F15" s="4">
         <v>2</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="H15" t="s">
         <v>389</v>
@@ -9246,13 +9302,13 @@
     </row>
     <row r="16" spans="1:13" ht="15">
       <c r="A16" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F16" s="4">
         <v>1</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H16" t="s">
         <v>389</v>
@@ -9260,16 +9316,16 @@
     </row>
     <row r="17" spans="1:8" ht="15">
       <c r="A17" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="F17" s="4">
         <v>1</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="H17" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="15">
@@ -9280,7 +9336,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="H18" t="s">
         <v>388</v>
@@ -9288,13 +9344,13 @@
     </row>
     <row r="19" spans="1:8" ht="15">
       <c r="A19" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="F19" s="4">
         <v>1</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="H19" t="s">
         <v>388</v>
@@ -9321,7 +9377,7 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="54" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="K1" t="s">
         <v>273</v>
@@ -9339,7 +9395,7 @@
     </row>
     <row r="5" spans="1:15">
       <c r="M5" s="53" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="N5" s="14"/>
       <c r="O5" s="14"/>
@@ -9349,7 +9405,7 @@
         <v>322</v>
       </c>
       <c r="M6" s="53" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="N6" s="14"/>
       <c r="O6" s="14"/>
@@ -9380,7 +9436,7 @@
       </c>
       <c r="C12" s="15"/>
       <c r="M12" s="53" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
       <c r="N12" s="14"/>
       <c r="O12" s="14"/>
@@ -9441,7 +9497,7 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="54" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="L1" t="s">
         <v>273</v>
@@ -9464,7 +9520,7 @@
         <v>365</v>
       </c>
       <c r="L4" s="53" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="M4" s="14"/>
       <c r="N4" s="14"/>
@@ -9472,7 +9528,7 @@
     <row r="5" spans="1:15">
       <c r="A5" s="54"/>
       <c r="L5" s="53" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="M5" s="14"/>
       <c r="N5" s="14"/>
@@ -9489,7 +9545,7 @@
         <v>246</v>
       </c>
       <c r="L7" s="53" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="M7" s="14"/>
       <c r="N7" s="14"/>
@@ -9512,10 +9568,10 @@
     <row r="10" spans="1:15">
       <c r="A10" s="54"/>
       <c r="C10" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="L10" s="53" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="M10" s="14"/>
       <c r="N10" s="14"/>
@@ -9710,22 +9766,22 @@
     </row>
     <row r="47" spans="2:2">
       <c r="B47" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="48" spans="2:2">
       <c r="B48" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="50" spans="2:2">
       <c r="B50" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="51" spans="2:2">
       <c r="B51" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="54" spans="2:2">
@@ -9801,7 +9857,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="I6" s="53" t="s">
-        <v>698</v>
+        <v>694</v>
       </c>
       <c r="J6" s="14"/>
       <c r="K6" s="14"/>
@@ -9811,14 +9867,14 @@
         <v>292</v>
       </c>
       <c r="I7" s="53" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="J7" s="14"/>
       <c r="K7" s="14"/>
     </row>
     <row r="8" spans="1:12">
       <c r="I8" s="53" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -9833,7 +9889,7 @@
         <v>294</v>
       </c>
       <c r="I10" s="53" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
@@ -9843,7 +9899,7 @@
         <v>295</v>
       </c>
       <c r="I11" s="53" t="s">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
@@ -9851,7 +9907,7 @@
     </row>
     <row r="12" spans="1:12">
       <c r="I12" s="53" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="J12" s="14"/>
       <c r="K12" s="14"/>
@@ -10036,12 +10092,12 @@
     </row>
     <row r="67" spans="2:8">
       <c r="B67" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="68" spans="2:8">
       <c r="B68" s="14" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="C68" s="14"/>
       <c r="D68" s="14"/>

</xml_diff>

<commit_message>
group_var split working - need to check no group and sorts
Former-commit-id: da044382b51340b8790955a5af6507db729f8652
</commit_message>
<xml_diff>
--- a/TestCampaign/ROVCleaver UniversalSetup.xlsx
+++ b/TestCampaign/ROVCleaver UniversalSetup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/PythonProgs/ROVCleaver_on_Dropbox/TestCampaign/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7EA7A98-7DF7-FB43-A5AC-A43167471E5C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D32D9D2-544C-6544-8511-43B942C5474B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25940" windowHeight="14100" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
   </bookViews>
@@ -518,7 +518,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1443" uniqueCount="718">
   <si>
     <t>File</t>
   </si>
@@ -2703,9 +2703,6 @@
     <t>Along with Factory fields, used to split concatenated file.  Most often County but can be other (eg, District) or a custom group created in modicode code (eg, age group such as "Over 50")</t>
   </si>
   <si>
-    <t>race,age</t>
-  </si>
-  <si>
     <t>Used to split at factory level if multiple factories are being loaded with addresses from one combined file.  Most often blank but can be other (eg, District) or a custom group created in modicode code (eg, age group such as "Over 50")</t>
   </si>
   <si>
@@ -2715,7 +2712,28 @@
     <t>False,("xl_factory_vars","str",{'str_case':'l'})</t>
   </si>
   <si>
-    <t>Almost always county (used to separate files for Sincere along with factory_vars)</t>
+    <t>age_group</t>
+  </si>
+  <si>
+    <t># make up fields for testing</t>
+  </si>
+  <si>
+    <t>Race,  Age_group</t>
+  </si>
+  <si>
+    <t>race</t>
+  </si>
+  <si>
+    <t>df['age_group'] = df['age'].map(lambda x: ('Young' if x &lt;50 else 'Senior') )</t>
+  </si>
+  <si>
+    <t>statecounty</t>
+  </si>
+  <si>
+    <t>Almost always statecounty (used to separate files for Sincere along with factory_vars)</t>
+  </si>
+  <si>
+    <t>df['race'] = df['rownum'].map(lambda x: ('Hispanic' if x % 2==0 else 'Black') )</t>
   </si>
 </sst>
 </file>
@@ -3090,7 +3108,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -3137,6 +3155,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3146,7 +3186,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
@@ -3257,7 +3297,6 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3294,8 +3333,15 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="4" builtinId="3"/>
@@ -3626,7 +3672,7 @@
     <col min="2" max="3" width="8.1640625" customWidth="1" outlineLevel="3"/>
     <col min="4" max="4" width="8.83203125" customWidth="1" outlineLevel="3"/>
     <col min="5" max="5" width="45" customWidth="1" outlineLevel="3"/>
-    <col min="6" max="6" width="38.6640625" style="81" customWidth="1" outlineLevel="2"/>
+    <col min="6" max="6" width="38.6640625" style="80" customWidth="1" outlineLevel="2"/>
     <col min="7" max="7" width="59.1640625" customWidth="1"/>
     <col min="8" max="8" width="14.6640625" customWidth="1"/>
     <col min="9" max="9" width="12.33203125" customWidth="1"/>
@@ -3650,13 +3696,13 @@
       <c r="E1" t="s">
         <v>463</v>
       </c>
-      <c r="F1" s="81" t="s">
+      <c r="F1" s="80" t="s">
         <v>483</v>
       </c>
       <c r="G1" s="64" t="s">
         <v>289</v>
       </c>
-      <c r="J1" s="87" t="s">
+      <c r="J1" s="86" t="s">
         <v>671</v>
       </c>
       <c r="K1" s="63"/>
@@ -3669,7 +3715,7 @@
       <c r="C2">
         <v>2</v>
       </c>
-      <c r="F2" s="82"/>
+      <c r="F2" s="81"/>
       <c r="G2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="21">
@@ -3715,7 +3761,7 @@
       <c r="E5" s="15" t="s">
         <v>465</v>
       </c>
-      <c r="F5" s="81" t="s">
+      <c r="F5" s="80" t="s">
         <v>645</v>
       </c>
       <c r="G5" s="65" t="s">
@@ -3769,7 +3815,7 @@
       <c r="E8" s="15" t="s">
         <v>466</v>
       </c>
-      <c r="F8" s="81" t="s">
+      <c r="F8" s="80" t="s">
         <v>646</v>
       </c>
       <c r="G8" s="65" t="s">
@@ -3814,7 +3860,7 @@
       <c r="E11" s="15" t="s">
         <v>507</v>
       </c>
-      <c r="F11" s="83" t="s">
+      <c r="F11" s="82" t="s">
         <v>647</v>
       </c>
       <c r="G11" s="65" t="s">
@@ -3860,7 +3906,7 @@
       <c r="E14" s="15" t="s">
         <v>508</v>
       </c>
-      <c r="F14" s="81" t="s">
+      <c r="F14" s="80" t="s">
         <v>648</v>
       </c>
       <c r="G14" s="65" t="s">
@@ -3904,16 +3950,16 @@
         <v>1</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>709</v>
-      </c>
-      <c r="F17" s="81" t="s">
+        <v>708</v>
+      </c>
+      <c r="F17" s="80" t="s">
         <v>706</v>
       </c>
       <c r="G17" s="67" t="s">
-        <v>19</v>
+        <v>715</v>
       </c>
       <c r="H17" s="66" t="s">
-        <v>711</v>
+        <v>716</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="16" thickTop="1">
@@ -3946,17 +3992,17 @@
       <c r="C20">
         <v>18.399999999999999</v>
       </c>
-      <c r="D20" s="92" t="b">
+      <c r="D20" s="90" t="b">
         <v>1</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>710</v>
-      </c>
-      <c r="F20" s="81" t="s">
-        <v>708</v>
+        <v>709</v>
+      </c>
+      <c r="F20" s="80" t="s">
+        <v>707</v>
       </c>
       <c r="G20" s="67" t="s">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="H20" s="66" t="s">
         <v>703</v>
@@ -3995,7 +4041,7 @@
       <c r="E23" s="15" t="s">
         <v>471</v>
       </c>
-      <c r="F23" s="83" t="s">
+      <c r="F23" s="82" t="s">
         <v>649</v>
       </c>
       <c r="G23" s="67">
@@ -4094,13 +4140,13 @@
       <c r="C31">
         <v>28</v>
       </c>
-      <c r="F31" s="81" t="s">
+      <c r="F31" s="80" t="s">
         <v>651</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="H31" s="88" t="s">
+      <c r="H31" s="87" t="s">
         <v>672</v>
       </c>
       <c r="L31" s="62" t="s">
@@ -4109,7 +4155,7 @@
       <c r="M31" s="62"/>
       <c r="N31" s="14"/>
     </row>
-    <row r="32" spans="1:14" ht="16" thickBot="1">
+    <row r="32" spans="1:14">
       <c r="B32">
         <v>14</v>
       </c>
@@ -4120,125 +4166,147 @@
         <v>597</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="17" thickTop="1" thickBot="1">
+    <row r="33" spans="1:29">
       <c r="A33" t="b">
         <v>1</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="90">
         <v>141</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="90">
         <v>30</v>
       </c>
-      <c r="D33" t="b">
-        <v>1</v>
-      </c>
-      <c r="E33" s="15" t="s">
+      <c r="D33" s="90" t="b">
+        <v>1</v>
+      </c>
+      <c r="E33" s="92" t="s">
         <v>468</v>
       </c>
-      <c r="F33" s="83" t="s">
+      <c r="F33" s="93" t="s">
         <v>533</v>
       </c>
-      <c r="G33" s="70" t="s">
+      <c r="G33" s="95" t="s">
         <v>348</v>
       </c>
-      <c r="H33" s="70" t="s">
+      <c r="H33" s="95" t="s">
         <v>201</v>
       </c>
-      <c r="I33" s="70" t="s">
+      <c r="I33" s="95" t="s">
         <v>204</v>
       </c>
-      <c r="J33" s="70" t="s">
+      <c r="J33" s="95" t="s">
         <v>205</v>
       </c>
-      <c r="K33" s="70" t="s">
+      <c r="K33" s="95" t="s">
         <v>206</v>
       </c>
-      <c r="L33" s="70" t="s">
+      <c r="L33" s="95" t="s">
         <v>48</v>
       </c>
-      <c r="M33" s="70" t="s">
+      <c r="M33" s="95" t="s">
         <v>207</v>
       </c>
-      <c r="N33" s="70" t="s">
+      <c r="N33" s="95" t="s">
         <v>208</v>
       </c>
-      <c r="O33" s="70" t="s">
+      <c r="O33" s="95" t="s">
         <v>209</v>
       </c>
-      <c r="P33" s="70" t="s">
+      <c r="P33" s="95" t="s">
         <v>210</v>
       </c>
-      <c r="Q33" s="71" t="s">
+      <c r="Q33" s="60" t="s">
         <v>211</v>
       </c>
-      <c r="R33" s="71"/>
-      <c r="S33" s="71"/>
-      <c r="T33" s="71"/>
-    </row>
-    <row r="34" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="R33" s="60"/>
+      <c r="S33" s="60"/>
+      <c r="T33" s="60"/>
+      <c r="U33" s="60"/>
+      <c r="V33" s="60"/>
+      <c r="W33" s="60"/>
+      <c r="X33" s="60"/>
+      <c r="Y33" s="60"/>
+      <c r="Z33" s="60"/>
+      <c r="AA33" s="60"/>
+      <c r="AB33" s="60"/>
+      <c r="AC33" s="60"/>
+    </row>
+    <row r="34" spans="1:29">
       <c r="A34" t="b">
         <v>1</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="90">
         <v>142</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="90">
         <v>31</v>
       </c>
-      <c r="D34" t="b">
-        <v>1</v>
-      </c>
-      <c r="E34" s="15" t="s">
+      <c r="D34" s="90" t="b">
+        <v>1</v>
+      </c>
+      <c r="E34" s="92" t="s">
         <v>469</v>
       </c>
-      <c r="F34" s="81" t="s">
+      <c r="F34" s="94" t="s">
         <v>277</v>
       </c>
-      <c r="G34" s="71" t="s">
+      <c r="G34" s="96" t="s">
         <v>348</v>
       </c>
-      <c r="H34" s="71" t="s">
+      <c r="H34" s="96" t="s">
         <v>20</v>
       </c>
-      <c r="I34" s="71" t="s">
+      <c r="I34" s="96" t="s">
         <v>22</v>
       </c>
-      <c r="J34" s="71" t="s">
+      <c r="J34" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="K34" s="71" t="s">
+      <c r="K34" s="96" t="s">
         <v>24</v>
       </c>
-      <c r="L34" s="71" t="s">
+      <c r="L34" s="96" t="s">
         <v>19</v>
       </c>
-      <c r="M34" s="71" t="s">
+      <c r="M34" s="96" t="s">
         <v>54</v>
       </c>
-      <c r="N34" s="71" t="s">
+      <c r="N34" s="96" t="s">
         <v>15</v>
       </c>
-      <c r="O34" s="71" t="s">
+      <c r="O34" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="P34" s="71" t="s">
+      <c r="P34" s="96" t="s">
         <v>17</v>
       </c>
-      <c r="Q34" s="71" t="s">
+      <c r="Q34" s="96" t="s">
         <v>21</v>
       </c>
-      <c r="R34" s="71" t="s">
+      <c r="R34" s="96" t="s">
         <v>14</v>
       </c>
-      <c r="S34" s="71" t="s">
+      <c r="S34" s="96" t="s">
         <v>378</v>
       </c>
-      <c r="T34" s="70" t="s">
+      <c r="T34" s="97" t="s">
         <v>556</v>
       </c>
-    </row>
-    <row r="35" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="U34" s="96" t="s">
+        <v>713</v>
+      </c>
+      <c r="V34" s="96" t="s">
+        <v>710</v>
+      </c>
+      <c r="W34" s="96"/>
+      <c r="X34" s="96"/>
+      <c r="Y34" s="96"/>
+      <c r="Z34" s="96"/>
+      <c r="AA34" s="96"/>
+      <c r="AB34" s="96"/>
+      <c r="AC34" s="96"/>
+    </row>
+    <row r="35" spans="1:29" ht="16" thickBot="1">
       <c r="A35" t="b">
         <v>1</v>
       </c>
@@ -4254,12 +4322,12 @@
       <c r="E35" s="15" t="s">
         <v>470</v>
       </c>
-      <c r="F35" s="83" t="s">
+      <c r="F35" s="82" t="s">
         <v>650</v>
       </c>
-      <c r="G35" s="79"/>
-      <c r="H35" s="80"/>
-      <c r="I35" s="80"/>
+      <c r="G35" s="78"/>
+      <c r="H35" s="79"/>
+      <c r="I35" s="79"/>
       <c r="J35" s="91" t="s">
         <v>270</v>
       </c>
@@ -4267,7 +4335,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="16" thickTop="1">
+    <row r="36" spans="1:29" ht="16" thickTop="1">
       <c r="B36">
         <v>149</v>
       </c>
@@ -4275,7 +4343,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="16" thickBot="1">
+    <row r="37" spans="1:29">
       <c r="B37">
         <v>150</v>
       </c>
@@ -4285,8 +4353,11 @@
       <c r="G37" s="1" t="s">
         <v>598</v>
       </c>
-    </row>
-    <row r="38" spans="1:20" ht="17" thickTop="1" thickBot="1">
+      <c r="H37" s="66" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="38" spans="1:29">
       <c r="A38" s="57" t="s">
         <v>490</v>
       </c>
@@ -4302,17 +4373,19 @@
       <c r="E38" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="F38" s="81" t="s">
+      <c r="F38" s="80" t="s">
         <v>666</v>
       </c>
-      <c r="G38" s="71" t="s">
+      <c r="G38" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="H38" s="66" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" ht="16" thickTop="1">
+      <c r="H38" s="98"/>
+      <c r="I38" s="98"/>
+      <c r="J38" s="98"/>
+      <c r="K38" s="98"/>
+      <c r="L38" s="98"/>
+    </row>
+    <row r="39" spans="1:29">
       <c r="B39">
         <v>152</v>
       </c>
@@ -4320,7 +4393,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="16" thickBot="1">
+    <row r="40" spans="1:29" ht="16" thickBot="1">
       <c r="B40">
         <v>155</v>
       </c>
@@ -4334,7 +4407,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="17" thickTop="1" thickBot="1">
+    <row r="41" spans="1:29" ht="17" thickTop="1" thickBot="1">
       <c r="A41" t="b">
         <v>1</v>
       </c>
@@ -4350,53 +4423,53 @@
       <c r="E41" s="15" t="s">
         <v>473</v>
       </c>
-      <c r="F41" s="81" t="s">
+      <c r="F41" s="80" t="s">
         <v>667</v>
       </c>
-      <c r="G41" s="71" t="s">
+      <c r="G41" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="H41" s="71" t="s">
+      <c r="H41" s="70" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="71" t="s">
+      <c r="I41" s="70" t="s">
         <v>14</v>
       </c>
-      <c r="J41" s="71" t="s">
+      <c r="J41" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="K41" s="71" t="s">
+      <c r="K41" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="L41" s="71" t="s">
+      <c r="L41" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="M41" s="71" t="s">
+      <c r="M41" s="70" t="s">
         <v>24</v>
       </c>
-      <c r="N41" s="71" t="s">
+      <c r="N41" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="O41" s="71" t="s">
+      <c r="O41" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="P41" s="71" t="s">
+      <c r="P41" s="70" t="s">
         <v>364</v>
       </c>
-      <c r="Q41" s="71" t="s">
+      <c r="Q41" s="70" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="16" thickTop="1">
+    <row r="42" spans="1:29" ht="16" thickTop="1">
       <c r="B42">
         <v>157</v>
       </c>
       <c r="C42">
         <v>39</v>
       </c>
-      <c r="F42" s="83"/>
-    </row>
-    <row r="43" spans="1:20" ht="16" thickBot="1">
+      <c r="F42" s="82"/>
+    </row>
+    <row r="43" spans="1:29" ht="16" thickBot="1">
       <c r="B43">
         <v>191</v>
       </c>
@@ -4407,7 +4480,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="17" thickTop="1" thickBot="1">
+    <row r="44" spans="1:29" ht="17" thickTop="1" thickBot="1">
       <c r="A44" s="57" t="s">
         <v>492</v>
       </c>
@@ -4423,17 +4496,17 @@
       <c r="E44" s="15" t="s">
         <v>510</v>
       </c>
-      <c r="F44" s="81" t="s">
+      <c r="F44" s="80" t="s">
         <v>279</v>
       </c>
-      <c r="G44" s="72" t="s">
+      <c r="G44" s="71" t="s">
         <v>348</v>
       </c>
       <c r="H44" s="66" t="s">
         <v>603</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="16" thickTop="1">
+    <row r="45" spans="1:29" ht="16" thickTop="1">
       <c r="B45">
         <v>193</v>
       </c>
@@ -4441,7 +4514,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="16" thickBot="1">
+    <row r="46" spans="1:29" ht="16" thickBot="1">
       <c r="B46">
         <v>194</v>
       </c>
@@ -4453,7 +4526,7 @@
       </c>
       <c r="H46" s="66"/>
     </row>
-    <row r="47" spans="1:20" ht="17" thickTop="1" thickBot="1">
+    <row r="47" spans="1:29" ht="17" thickTop="1" thickBot="1">
       <c r="A47" s="57" t="s">
         <v>493</v>
       </c>
@@ -4469,14 +4542,14 @@
       <c r="E47" s="15" t="s">
         <v>511</v>
       </c>
-      <c r="F47" s="81" t="s">
+      <c r="F47" s="80" t="s">
         <v>278</v>
       </c>
-      <c r="G47" s="72" t="s">
+      <c r="G47" s="71" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="16" thickTop="1">
+    <row r="48" spans="1:29" ht="16" thickTop="1">
       <c r="B48">
         <v>196</v>
       </c>
@@ -4511,10 +4584,10 @@
       <c r="E50" s="15" t="s">
         <v>509</v>
       </c>
-      <c r="F50" s="81" t="s">
+      <c r="F50" s="80" t="s">
         <v>652</v>
       </c>
-      <c r="G50" s="73" t="b">
+      <c r="G50" s="72" t="b">
         <v>0</v>
       </c>
       <c r="H50" s="66" t="s">
@@ -4544,7 +4617,7 @@
       </c>
     </row>
     <row r="53" spans="1:16" ht="49" thickBot="1">
-      <c r="B53" s="78">
+      <c r="B53" s="77">
         <v>97.5</v>
       </c>
       <c r="C53">
@@ -4576,16 +4649,16 @@
       <c r="E54" s="15" t="s">
         <v>525</v>
       </c>
-      <c r="F54" s="81" t="s">
+      <c r="F54" s="80" t="s">
         <v>535</v>
       </c>
-      <c r="G54" s="72" t="s">
+      <c r="G54" s="71" t="s">
         <v>387</v>
       </c>
-      <c r="H54" s="74" t="b">
+      <c r="H54" s="73" t="b">
         <v>0</v>
       </c>
-      <c r="I54" s="72" t="b">
+      <c r="I54" s="71" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4605,12 +4678,12 @@
       <c r="E55" s="15" t="s">
         <v>526</v>
       </c>
-      <c r="F55" s="83"/>
-      <c r="G55" s="72"/>
-      <c r="H55" s="72" t="b">
+      <c r="F55" s="82"/>
+      <c r="G55" s="71"/>
+      <c r="H55" s="71" t="b">
         <v>0</v>
       </c>
-      <c r="I55" s="72" t="b">
+      <c r="I55" s="71" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4630,13 +4703,13 @@
       <c r="E56" s="15" t="s">
         <v>527</v>
       </c>
-      <c r="G56" s="72" t="s">
+      <c r="G56" s="71" t="s">
         <v>455</v>
       </c>
-      <c r="H56" s="72" t="b">
+      <c r="H56" s="71" t="b">
         <v>0</v>
       </c>
-      <c r="I56" s="72" t="b">
+      <c r="I56" s="71" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4656,13 +4729,13 @@
       <c r="E57" s="15" t="s">
         <v>528</v>
       </c>
-      <c r="G57" s="72" t="s">
+      <c r="G57" s="71" t="s">
         <v>390</v>
       </c>
-      <c r="H57" s="72" t="b">
-        <v>1</v>
-      </c>
-      <c r="I57" s="72" t="b">
+      <c r="H57" s="71" t="b">
+        <v>1</v>
+      </c>
+      <c r="I57" s="71" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4682,13 +4755,13 @@
       <c r="E58" s="15" t="s">
         <v>529</v>
       </c>
-      <c r="G58" s="72" t="s">
+      <c r="G58" s="71" t="s">
         <v>544</v>
       </c>
-      <c r="H58" s="72" t="b">
+      <c r="H58" s="71" t="b">
         <v>0</v>
       </c>
-      <c r="I58" s="72" t="b">
+      <c r="I58" s="71" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4754,10 +4827,10 @@
       <c r="E63" t="s">
         <v>472</v>
       </c>
-      <c r="F63" s="81" t="s">
+      <c r="F63" s="80" t="s">
         <v>655</v>
       </c>
-      <c r="G63" s="72" t="s">
+      <c r="G63" s="71" t="s">
         <v>276</v>
       </c>
       <c r="H63" s="66" t="s">
@@ -4799,10 +4872,10 @@
       <c r="E66" s="15" t="s">
         <v>505</v>
       </c>
-      <c r="F66" s="81" t="s">
+      <c r="F66" s="80" t="s">
         <v>531</v>
       </c>
-      <c r="G66" s="73">
+      <c r="G66" s="72">
         <v>3</v>
       </c>
       <c r="H66" s="66" t="s">
@@ -4853,7 +4926,7 @@
       <c r="E69" s="15" t="s">
         <v>536</v>
       </c>
-      <c r="F69" s="81" t="s">
+      <c r="F69" s="80" t="s">
         <v>657</v>
       </c>
       <c r="G69" t="s">
@@ -4878,12 +4951,12 @@
       <c r="G71" s="32" t="s">
         <v>660</v>
       </c>
-      <c r="H71" s="84" t="s">
+      <c r="H71" s="83" t="s">
         <v>661</v>
       </c>
       <c r="I71" s="14"/>
-      <c r="J71" s="79"/>
-      <c r="K71" s="79"/>
+      <c r="J71" s="78"/>
+      <c r="K71" s="78"/>
       <c r="L71" s="62" t="s">
         <v>669</v>
       </c>
@@ -4907,10 +4980,10 @@
       <c r="E72" s="15" t="s">
         <v>481</v>
       </c>
-      <c r="F72" s="81" t="s">
+      <c r="F72" s="80" t="s">
         <v>542</v>
       </c>
-      <c r="G72" s="72" t="s">
+      <c r="G72" s="71" t="s">
         <v>482</v>
       </c>
       <c r="L72" s="62" t="s">
@@ -4955,10 +5028,10 @@
       <c r="E75" s="15" t="s">
         <v>512</v>
       </c>
-      <c r="F75" s="81" t="s">
+      <c r="F75" s="80" t="s">
         <v>668</v>
       </c>
-      <c r="G75" s="73" t="b">
+      <c r="G75" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H75" s="66" t="s">
@@ -5005,10 +5078,10 @@
       <c r="E78" s="15" t="s">
         <v>513</v>
       </c>
-      <c r="F78" s="85" t="s">
+      <c r="F78" s="84" t="s">
         <v>534</v>
       </c>
-      <c r="G78" s="73" t="b">
+      <c r="G78" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H78" s="66" t="s">
@@ -5050,10 +5123,10 @@
       <c r="E81" s="15" t="s">
         <v>521</v>
       </c>
-      <c r="F81" s="81" t="s">
+      <c r="F81" s="80" t="s">
         <v>662</v>
       </c>
-      <c r="G81" s="73" t="s">
+      <c r="G81" s="72" t="s">
         <v>196</v>
       </c>
       <c r="H81" s="66" t="s">
@@ -5114,10 +5187,10 @@
       <c r="E86" s="15" t="s">
         <v>514</v>
       </c>
-      <c r="F86" s="81" t="s">
+      <c r="F86" s="80" t="s">
         <v>663</v>
       </c>
-      <c r="G86" s="73" t="b">
+      <c r="G86" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H86" s="66" t="s">
@@ -5160,10 +5233,10 @@
       <c r="E89" s="15" t="s">
         <v>515</v>
       </c>
-      <c r="F89" s="81" t="s">
+      <c r="F89" s="80" t="s">
         <v>664</v>
       </c>
-      <c r="G89" s="73" t="b">
+      <c r="G89" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H89" s="66" t="s">
@@ -5185,7 +5258,7 @@
       <c r="C91">
         <v>88</v>
       </c>
-      <c r="G91" s="86" t="s">
+      <c r="G91" s="85" t="s">
         <v>329</v>
       </c>
       <c r="N91" s="62" t="s">
@@ -5212,10 +5285,10 @@
       <c r="E92" s="15" t="s">
         <v>517</v>
       </c>
-      <c r="F92" s="85" t="s">
+      <c r="F92" s="84" t="s">
         <v>532</v>
       </c>
-      <c r="G92" s="75">
+      <c r="G92" s="74">
         <v>3</v>
       </c>
       <c r="H92" s="66" t="s">
@@ -5229,7 +5302,7 @@
       <c r="C93">
         <v>90</v>
       </c>
-      <c r="G93" s="76" t="s">
+      <c r="G93" s="75" t="s">
         <v>266</v>
       </c>
       <c r="L93" s="62" t="s">
@@ -5274,17 +5347,17 @@
       <c r="E96" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="F96" s="81" t="s">
+      <c r="F96" s="80" t="s">
         <v>670</v>
       </c>
-      <c r="G96" s="75">
+      <c r="G96" s="74">
         <v>25000</v>
       </c>
       <c r="H96" s="66" t="s">
         <v>631</v>
       </c>
-      <c r="J96" s="76"/>
-      <c r="K96" s="76"/>
+      <c r="J96" s="75"/>
+      <c r="K96" s="75"/>
     </row>
     <row r="97" spans="1:16" ht="16" thickTop="1">
       <c r="B97">
@@ -5323,10 +5396,10 @@
       <c r="G100" s="1" t="s">
         <v>632</v>
       </c>
-      <c r="H100" s="89" t="s">
+      <c r="H100" s="88" t="s">
         <v>674</v>
       </c>
-      <c r="I100" s="79"/>
+      <c r="I100" s="78"/>
     </row>
     <row r="101" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A101" t="s">
@@ -5344,10 +5417,10 @@
       <c r="E101" s="15" t="s">
         <v>475</v>
       </c>
-      <c r="F101" s="81" t="s">
+      <c r="F101" s="80" t="s">
         <v>673</v>
       </c>
-      <c r="G101" s="73" t="b">
+      <c r="G101" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H101" s="66" t="s">
@@ -5382,26 +5455,26 @@
         <v>634</v>
       </c>
     </row>
-    <row r="104" spans="1:16" s="81" customFormat="1" ht="17" thickTop="1" thickBot="1">
-      <c r="A104" s="81" t="s">
+    <row r="104" spans="1:16" s="80" customFormat="1" ht="17" thickTop="1" thickBot="1">
+      <c r="A104" s="80" t="s">
         <v>480</v>
       </c>
-      <c r="B104" s="81">
+      <c r="B104" s="80">
         <v>224</v>
       </c>
       <c r="C104">
         <v>101</v>
       </c>
-      <c r="D104" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="E104" s="83" t="s">
+      <c r="D104" s="80" t="b">
+        <v>1</v>
+      </c>
+      <c r="E104" s="82" t="s">
         <v>522</v>
       </c>
-      <c r="F104" s="90" t="s">
+      <c r="F104" s="89" t="s">
         <v>675</v>
       </c>
-      <c r="G104" s="72" t="s">
+      <c r="G104" s="71" t="s">
         <v>284</v>
       </c>
       <c r="H104" s="66" t="s">
@@ -5453,10 +5526,10 @@
       <c r="E107" s="15" t="s">
         <v>476</v>
       </c>
-      <c r="F107" s="90" t="s">
+      <c r="F107" s="89" t="s">
         <v>676</v>
       </c>
-      <c r="G107" s="73" t="b">
+      <c r="G107" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H107" s="66" t="s">
@@ -5498,10 +5571,10 @@
       <c r="E110" s="15" t="s">
         <v>523</v>
       </c>
-      <c r="F110" s="90" t="s">
+      <c r="F110" s="89" t="s">
         <v>683</v>
       </c>
-      <c r="G110" s="72" t="s">
+      <c r="G110" s="71" t="s">
         <v>285</v>
       </c>
       <c r="H110" s="66" t="s">
@@ -5553,10 +5626,10 @@
       <c r="E113" s="15" t="s">
         <v>479</v>
       </c>
-      <c r="F113" s="90" t="s">
+      <c r="F113" s="89" t="s">
         <v>680</v>
       </c>
-      <c r="G113" s="73" t="b">
+      <c r="G113" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H113" s="66" t="s">
@@ -5598,10 +5671,10 @@
       <c r="E116" s="15" t="s">
         <v>524</v>
       </c>
-      <c r="F116" s="90" t="s">
+      <c r="F116" s="89" t="s">
         <v>681</v>
       </c>
-      <c r="G116" s="72" t="s">
+      <c r="G116" s="71" t="s">
         <v>286</v>
       </c>
       <c r="H116" s="66" t="s">
@@ -5669,10 +5742,10 @@
       <c r="E121" s="15" t="s">
         <v>516</v>
       </c>
-      <c r="F121" s="90" t="s">
+      <c r="F121" s="89" t="s">
         <v>686</v>
       </c>
-      <c r="G121" s="73" t="b">
+      <c r="G121" s="72" t="b">
         <v>0</v>
       </c>
       <c r="H121" s="66" t="s">
@@ -5686,7 +5759,7 @@
       <c r="C122">
         <v>119</v>
       </c>
-      <c r="G122" s="76"/>
+      <c r="G122" s="75"/>
     </row>
     <row r="123" spans="1:16" ht="16" thickBot="1">
       <c r="B123">
@@ -5695,7 +5768,7 @@
       <c r="C123">
         <v>120</v>
       </c>
-      <c r="G123" s="86" t="s">
+      <c r="G123" s="85" t="s">
         <v>192</v>
       </c>
     </row>
@@ -5715,10 +5788,10 @@
       <c r="E124" s="15" t="s">
         <v>537</v>
       </c>
-      <c r="F124" s="85" t="s">
+      <c r="F124" s="84" t="s">
         <v>539</v>
       </c>
-      <c r="G124" s="71" t="s">
+      <c r="G124" s="70" t="s">
         <v>193</v>
       </c>
     </row>
@@ -5737,10 +5810,10 @@
       <c r="C126">
         <v>123</v>
       </c>
-      <c r="G126" s="86" t="s">
+      <c r="G126" s="85" t="s">
         <v>665</v>
       </c>
-      <c r="N126" s="77" t="s">
+      <c r="N126" s="76" t="s">
         <v>643</v>
       </c>
       <c r="O126" s="61"/>
@@ -5762,10 +5835,10 @@
       <c r="E127" s="15" t="s">
         <v>538</v>
       </c>
-      <c r="F127" s="85" t="s">
+      <c r="F127" s="84" t="s">
         <v>540</v>
       </c>
-      <c r="G127" s="71" t="s">
+      <c r="G127" s="70" t="s">
         <v>191</v>
       </c>
     </row>
@@ -5814,7 +5887,7 @@
       <c r="E130" s="15" t="s">
         <v>520</v>
       </c>
-      <c r="F130" s="81" t="s">
+      <c r="F130" s="80" t="s">
         <v>280</v>
       </c>
       <c r="G130" t="s">
@@ -9136,7 +9209,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>549</v>
@@ -9155,6 +9228,9 @@
       <c r="C6" s="4" t="s">
         <v>1</v>
       </c>
+      <c r="F6" s="4">
+        <v>3</v>
+      </c>
       <c r="G6" s="4" t="s">
         <v>550</v>
       </c>
@@ -9185,12 +9261,6 @@
     <row r="8" spans="1:13" ht="15">
       <c r="A8" t="s">
         <v>386</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>1</v>
       </c>
       <c r="F8" s="4">
         <v>4</v>
@@ -9489,7 +9559,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2646F8F-FCED-7B48-A04F-8BFFB0821CB1}">
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="11" width="6.33203125" customWidth="1"/>
@@ -9817,6 +9887,21 @@
     <row r="63" spans="2:2">
       <c r="B63" t="s">
         <v>363</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2">
+      <c r="B66" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2">
+      <c r="B67" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2">
+      <c r="B68" t="s">
+        <v>717</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hardcoded paths to raw zip csvs to accommodate cleaver_prod and _test
Former-commit-id: e006184567f91057662550d517ab2a395e6ca282
</commit_message>
<xml_diff>
--- a/TestCampaign/ROVCleaver UniversalSetup.xlsx
+++ b/TestCampaign/ROVCleaver UniversalSetup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/PythonProgs/ROVCleaver_on_Dropbox/TestCampaign/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D32D9D2-544C-6544-8511-43B942C5474B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D208213-AC05-E647-AFFB-D47B5A35152A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25940" windowHeight="14100" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
   </bookViews>
@@ -3156,25 +3156,23 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top/>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
       <bottom style="thick">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="thin">
+      <top style="thick">
         <color auto="1"/>
-      </bottom>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -3186,7 +3184,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
@@ -3314,7 +3312,6 @@
     <xf numFmtId="0" fontId="41" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
@@ -3334,14 +3331,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="4" builtinId="3"/>
@@ -3665,14 +3664,14 @@
     <tabColor rgb="FFFFFF00"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AD194"/>
+  <dimension ref="A1:AE194"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1" outlineLevel="3"/>
-    <col min="2" max="3" width="8.1640625" customWidth="1" outlineLevel="3"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1" outlineLevel="3"/>
-    <col min="5" max="5" width="45" customWidth="1" outlineLevel="3"/>
-    <col min="6" max="6" width="38.6640625" style="80" customWidth="1" outlineLevel="2"/>
+    <col min="1" max="1" width="10" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="2" max="3" width="8.1640625" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="4" max="4" width="8.83203125" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="5" max="5" width="45" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="6" max="6" width="38.6640625" style="79" customWidth="1" outlineLevel="2" collapsed="1"/>
     <col min="7" max="7" width="59.1640625" customWidth="1"/>
     <col min="8" max="8" width="14.6640625" customWidth="1"/>
     <col min="9" max="9" width="12.33203125" customWidth="1"/>
@@ -3696,13 +3695,13 @@
       <c r="E1" t="s">
         <v>463</v>
       </c>
-      <c r="F1" s="80" t="s">
+      <c r="F1" s="79" t="s">
         <v>483</v>
       </c>
       <c r="G1" s="64" t="s">
         <v>289</v>
       </c>
-      <c r="J1" s="86" t="s">
+      <c r="J1" s="85" t="s">
         <v>671</v>
       </c>
       <c r="K1" s="63"/>
@@ -3715,7 +3714,7 @@
       <c r="C2">
         <v>2</v>
       </c>
-      <c r="F2" s="81"/>
+      <c r="F2" s="80"/>
       <c r="G2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="21">
@@ -3761,7 +3760,7 @@
       <c r="E5" s="15" t="s">
         <v>465</v>
       </c>
-      <c r="F5" s="80" t="s">
+      <c r="F5" s="79" t="s">
         <v>645</v>
       </c>
       <c r="G5" s="65" t="s">
@@ -3815,7 +3814,7 @@
       <c r="E8" s="15" t="s">
         <v>466</v>
       </c>
-      <c r="F8" s="80" t="s">
+      <c r="F8" s="79" t="s">
         <v>646</v>
       </c>
       <c r="G8" s="65" t="s">
@@ -3860,7 +3859,7 @@
       <c r="E11" s="15" t="s">
         <v>507</v>
       </c>
-      <c r="F11" s="82" t="s">
+      <c r="F11" s="81" t="s">
         <v>647</v>
       </c>
       <c r="G11" s="65" t="s">
@@ -3906,7 +3905,7 @@
       <c r="E14" s="15" t="s">
         <v>508</v>
       </c>
-      <c r="F14" s="80" t="s">
+      <c r="F14" s="79" t="s">
         <v>648</v>
       </c>
       <c r="G14" s="65" t="s">
@@ -3952,7 +3951,7 @@
       <c r="E17" s="15" t="s">
         <v>708</v>
       </c>
-      <c r="F17" s="80" t="s">
+      <c r="F17" s="79" t="s">
         <v>706</v>
       </c>
       <c r="G17" s="67" t="s">
@@ -3992,13 +3991,13 @@
       <c r="C20">
         <v>18.399999999999999</v>
       </c>
-      <c r="D20" s="90" t="b">
+      <c r="D20" s="89" t="b">
         <v>1</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>709</v>
       </c>
-      <c r="F20" s="80" t="s">
+      <c r="F20" s="79" t="s">
         <v>707</v>
       </c>
       <c r="G20" s="67" t="s">
@@ -4041,7 +4040,7 @@
       <c r="E23" s="15" t="s">
         <v>471</v>
       </c>
-      <c r="F23" s="82" t="s">
+      <c r="F23" s="81" t="s">
         <v>649</v>
       </c>
       <c r="G23" s="67">
@@ -4140,13 +4139,13 @@
       <c r="C31">
         <v>28</v>
       </c>
-      <c r="F31" s="80" t="s">
+      <c r="F31" s="79" t="s">
         <v>651</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="H31" s="87" t="s">
+      <c r="H31" s="86" t="s">
         <v>672</v>
       </c>
       <c r="L31" s="62" t="s">
@@ -4155,7 +4154,7 @@
       <c r="M31" s="62"/>
       <c r="N31" s="14"/>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" ht="16" thickBot="1">
       <c r="B32">
         <v>14</v>
       </c>
@@ -4166,23 +4165,23 @@
         <v>597</v>
       </c>
     </row>
-    <row r="33" spans="1:29">
+    <row r="33" spans="1:31" ht="16" thickTop="1">
       <c r="A33" t="b">
         <v>1</v>
       </c>
-      <c r="B33" s="90">
+      <c r="B33" s="89">
         <v>141</v>
       </c>
-      <c r="C33" s="90">
+      <c r="C33" s="89">
         <v>30</v>
       </c>
-      <c r="D33" s="90" t="b">
-        <v>1</v>
-      </c>
-      <c r="E33" s="92" t="s">
+      <c r="D33" s="89" t="b">
+        <v>1</v>
+      </c>
+      <c r="E33" s="90" t="s">
         <v>468</v>
       </c>
-      <c r="F33" s="93" t="s">
+      <c r="F33" s="91" t="s">
         <v>533</v>
       </c>
       <c r="G33" s="95" t="s">
@@ -4215,98 +4214,102 @@
       <c r="P33" s="95" t="s">
         <v>210</v>
       </c>
-      <c r="Q33" s="60" t="s">
+      <c r="Q33" s="96" t="s">
         <v>211</v>
       </c>
-      <c r="R33" s="60"/>
-      <c r="S33" s="60"/>
-      <c r="T33" s="60"/>
-      <c r="U33" s="60"/>
-      <c r="V33" s="60"/>
-      <c r="W33" s="60"/>
-      <c r="X33" s="60"/>
-      <c r="Y33" s="60"/>
-      <c r="Z33" s="60"/>
-      <c r="AA33" s="60"/>
-      <c r="AB33" s="60"/>
-      <c r="AC33" s="60"/>
-    </row>
-    <row r="34" spans="1:29">
+      <c r="R33" s="96"/>
+      <c r="S33" s="96"/>
+      <c r="T33" s="96"/>
+      <c r="U33" s="96"/>
+      <c r="V33" s="96"/>
+      <c r="W33" s="96"/>
+      <c r="X33" s="96"/>
+      <c r="Y33" s="96"/>
+      <c r="Z33" s="96"/>
+      <c r="AA33" s="96"/>
+      <c r="AB33" s="96"/>
+      <c r="AC33" s="96"/>
+      <c r="AD33" s="96"/>
+      <c r="AE33" s="96"/>
+    </row>
+    <row r="34" spans="1:31" ht="16" thickBot="1">
       <c r="A34" t="b">
         <v>1</v>
       </c>
-      <c r="B34" s="90">
+      <c r="B34" s="89">
         <v>142</v>
       </c>
-      <c r="C34" s="90">
+      <c r="C34" s="89">
         <v>31</v>
       </c>
-      <c r="D34" s="90" t="b">
-        <v>1</v>
-      </c>
-      <c r="E34" s="92" t="s">
+      <c r="D34" s="89" t="b">
+        <v>1</v>
+      </c>
+      <c r="E34" s="90" t="s">
         <v>469</v>
       </c>
-      <c r="F34" s="94" t="s">
+      <c r="F34" s="93" t="s">
         <v>277</v>
       </c>
-      <c r="G34" s="96" t="s">
+      <c r="G34" s="89" t="s">
         <v>348</v>
       </c>
-      <c r="H34" s="96" t="s">
+      <c r="H34" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="I34" s="96" t="s">
+      <c r="I34" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="J34" s="96" t="s">
+      <c r="J34" s="89" t="s">
         <v>23</v>
       </c>
-      <c r="K34" s="96" t="s">
+      <c r="K34" s="89" t="s">
         <v>24</v>
       </c>
-      <c r="L34" s="96" t="s">
+      <c r="L34" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="M34" s="96" t="s">
+      <c r="M34" s="89" t="s">
         <v>54</v>
       </c>
-      <c r="N34" s="96" t="s">
+      <c r="N34" s="89" t="s">
         <v>15</v>
       </c>
-      <c r="O34" s="96" t="s">
+      <c r="O34" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="P34" s="96" t="s">
+      <c r="P34" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="Q34" s="96" t="s">
+      <c r="Q34" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="R34" s="96" t="s">
+      <c r="R34" s="89" t="s">
         <v>14</v>
       </c>
-      <c r="S34" s="96" t="s">
+      <c r="S34" s="89" t="s">
         <v>378</v>
       </c>
-      <c r="T34" s="97" t="s">
+      <c r="T34" s="92" t="s">
         <v>556</v>
       </c>
-      <c r="U34" s="96" t="s">
+      <c r="U34" s="89" t="s">
         <v>713</v>
       </c>
-      <c r="V34" s="96" t="s">
+      <c r="V34" s="89" t="s">
         <v>710</v>
       </c>
-      <c r="W34" s="96"/>
-      <c r="X34" s="96"/>
-      <c r="Y34" s="96"/>
-      <c r="Z34" s="96"/>
-      <c r="AA34" s="96"/>
-      <c r="AB34" s="96"/>
-      <c r="AC34" s="96"/>
-    </row>
-    <row r="35" spans="1:29" ht="16" thickBot="1">
+      <c r="W34" s="89"/>
+      <c r="X34" s="89"/>
+      <c r="Y34" s="89"/>
+      <c r="Z34" s="89"/>
+      <c r="AA34" s="89"/>
+      <c r="AB34" s="89"/>
+      <c r="AC34" s="89"/>
+      <c r="AD34" s="89"/>
+      <c r="AE34" s="89"/>
+    </row>
+    <row r="35" spans="1:31" ht="17" thickTop="1" thickBot="1">
       <c r="A35" t="b">
         <v>1</v>
       </c>
@@ -4322,20 +4325,40 @@
       <c r="E35" s="15" t="s">
         <v>470</v>
       </c>
-      <c r="F35" s="82" t="s">
+      <c r="F35" s="81" t="s">
         <v>650</v>
       </c>
-      <c r="G35" s="78"/>
-      <c r="H35" s="79"/>
-      <c r="I35" s="79"/>
-      <c r="J35" s="91" t="s">
+      <c r="G35" s="97"/>
+      <c r="H35" s="98"/>
+      <c r="I35" s="98"/>
+      <c r="J35" s="99" t="s">
         <v>270</v>
       </c>
-      <c r="K35" t="s">
+      <c r="K35" s="94" t="s">
         <v>692</v>
       </c>
-    </row>
-    <row r="36" spans="1:29" ht="16" thickTop="1">
+      <c r="L35" s="94"/>
+      <c r="M35" s="94"/>
+      <c r="N35" s="94"/>
+      <c r="O35" s="94"/>
+      <c r="P35" s="94"/>
+      <c r="Q35" s="94"/>
+      <c r="R35" s="94"/>
+      <c r="S35" s="94"/>
+      <c r="T35" s="94"/>
+      <c r="U35" s="94"/>
+      <c r="V35" s="94"/>
+      <c r="W35" s="94"/>
+      <c r="X35" s="94"/>
+      <c r="Y35" s="94"/>
+      <c r="Z35" s="94"/>
+      <c r="AA35" s="94"/>
+      <c r="AB35" s="94"/>
+      <c r="AC35" s="94"/>
+      <c r="AD35" s="94"/>
+      <c r="AE35" s="94"/>
+    </row>
+    <row r="36" spans="1:31" ht="16" thickTop="1">
       <c r="B36">
         <v>149</v>
       </c>
@@ -4343,7 +4366,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:29">
+    <row r="37" spans="1:31" ht="16" thickBot="1">
       <c r="B37">
         <v>150</v>
       </c>
@@ -4357,7 +4380,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="38" spans="1:29">
+    <row r="38" spans="1:31" ht="17" thickTop="1" thickBot="1">
       <c r="A38" s="57" t="s">
         <v>490</v>
       </c>
@@ -4373,19 +4396,24 @@
       <c r="E38" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="F38" s="80" t="s">
+      <c r="F38" s="79" t="s">
         <v>666</v>
       </c>
-      <c r="G38" s="98" t="s">
+      <c r="G38" s="94" t="s">
         <v>54</v>
       </c>
-      <c r="H38" s="98"/>
-      <c r="I38" s="98"/>
-      <c r="J38" s="98"/>
-      <c r="K38" s="98"/>
-      <c r="L38" s="98"/>
-    </row>
-    <row r="39" spans="1:29">
+      <c r="H38" s="94"/>
+      <c r="I38" s="94"/>
+      <c r="J38" s="94"/>
+      <c r="K38" s="94"/>
+      <c r="L38" s="94"/>
+      <c r="M38" s="94"/>
+      <c r="N38" s="94"/>
+      <c r="O38" s="94"/>
+      <c r="P38" s="94"/>
+      <c r="Q38" s="94"/>
+    </row>
+    <row r="39" spans="1:31" ht="16" thickTop="1">
       <c r="B39">
         <v>152</v>
       </c>
@@ -4393,7 +4421,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="40" spans="1:29" ht="16" thickBot="1">
+    <row r="40" spans="1:31" ht="16" thickBot="1">
       <c r="B40">
         <v>155</v>
       </c>
@@ -4407,7 +4435,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="41" spans="1:29" ht="17" thickTop="1" thickBot="1">
+    <row r="41" spans="1:31" ht="17" thickTop="1" thickBot="1">
       <c r="A41" t="b">
         <v>1</v>
       </c>
@@ -4423,53 +4451,59 @@
       <c r="E41" s="15" t="s">
         <v>473</v>
       </c>
-      <c r="F41" s="80" t="s">
+      <c r="F41" s="79" t="s">
         <v>667</v>
       </c>
-      <c r="G41" s="70" t="s">
+      <c r="G41" s="94" t="s">
         <v>20</v>
       </c>
-      <c r="H41" s="70" t="s">
+      <c r="H41" s="94" t="s">
         <v>22</v>
       </c>
-      <c r="I41" s="70" t="s">
+      <c r="I41" s="94" t="s">
         <v>14</v>
       </c>
-      <c r="J41" s="70" t="s">
+      <c r="J41" s="94" t="s">
         <v>16</v>
       </c>
-      <c r="K41" s="70" t="s">
+      <c r="K41" s="94" t="s">
         <v>21</v>
       </c>
-      <c r="L41" s="70" t="s">
+      <c r="L41" s="94" t="s">
         <v>17</v>
       </c>
-      <c r="M41" s="70" t="s">
+      <c r="M41" s="94" t="s">
         <v>24</v>
       </c>
-      <c r="N41" s="70" t="s">
+      <c r="N41" s="94" t="s">
         <v>23</v>
       </c>
-      <c r="O41" s="70" t="s">
+      <c r="O41" s="94" t="s">
         <v>19</v>
       </c>
-      <c r="P41" s="70" t="s">
+      <c r="P41" s="94" t="s">
         <v>364</v>
       </c>
-      <c r="Q41" s="70" t="s">
+      <c r="Q41" s="94" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="42" spans="1:29" ht="16" thickTop="1">
+      <c r="R41" s="94"/>
+      <c r="S41" s="94"/>
+      <c r="T41" s="94"/>
+      <c r="U41" s="94"/>
+      <c r="V41" s="94"/>
+      <c r="W41" s="94"/>
+    </row>
+    <row r="42" spans="1:31" ht="16" thickTop="1">
       <c r="B42">
         <v>157</v>
       </c>
       <c r="C42">
         <v>39</v>
       </c>
-      <c r="F42" s="82"/>
-    </row>
-    <row r="43" spans="1:29" ht="16" thickBot="1">
+      <c r="F42" s="81"/>
+    </row>
+    <row r="43" spans="1:31" ht="16" thickBot="1">
       <c r="B43">
         <v>191</v>
       </c>
@@ -4480,7 +4514,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="44" spans="1:29" ht="17" thickTop="1" thickBot="1">
+    <row r="44" spans="1:31" ht="17" thickTop="1" thickBot="1">
       <c r="A44" s="57" t="s">
         <v>492</v>
       </c>
@@ -4496,7 +4530,7 @@
       <c r="E44" s="15" t="s">
         <v>510</v>
       </c>
-      <c r="F44" s="80" t="s">
+      <c r="F44" s="79" t="s">
         <v>279</v>
       </c>
       <c r="G44" s="71" t="s">
@@ -4506,7 +4540,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="45" spans="1:29" ht="16" thickTop="1">
+    <row r="45" spans="1:31" ht="16" thickTop="1">
       <c r="B45">
         <v>193</v>
       </c>
@@ -4514,7 +4548,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:29" ht="16" thickBot="1">
+    <row r="46" spans="1:31" ht="16" thickBot="1">
       <c r="B46">
         <v>194</v>
       </c>
@@ -4526,7 +4560,7 @@
       </c>
       <c r="H46" s="66"/>
     </row>
-    <row r="47" spans="1:29" ht="17" thickTop="1" thickBot="1">
+    <row r="47" spans="1:31" ht="17" thickTop="1" thickBot="1">
       <c r="A47" s="57" t="s">
         <v>493</v>
       </c>
@@ -4542,14 +4576,14 @@
       <c r="E47" s="15" t="s">
         <v>511</v>
       </c>
-      <c r="F47" s="80" t="s">
+      <c r="F47" s="79" t="s">
         <v>278</v>
       </c>
       <c r="G47" s="71" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="48" spans="1:29" ht="16" thickTop="1">
+    <row r="48" spans="1:31" ht="16" thickTop="1">
       <c r="B48">
         <v>196</v>
       </c>
@@ -4584,7 +4618,7 @@
       <c r="E50" s="15" t="s">
         <v>509</v>
       </c>
-      <c r="F50" s="80" t="s">
+      <c r="F50" s="79" t="s">
         <v>652</v>
       </c>
       <c r="G50" s="72" t="b">
@@ -4649,7 +4683,7 @@
       <c r="E54" s="15" t="s">
         <v>525</v>
       </c>
-      <c r="F54" s="80" t="s">
+      <c r="F54" s="79" t="s">
         <v>535</v>
       </c>
       <c r="G54" s="71" t="s">
@@ -4678,7 +4712,7 @@
       <c r="E55" s="15" t="s">
         <v>526</v>
       </c>
-      <c r="F55" s="82"/>
+      <c r="F55" s="81"/>
       <c r="G55" s="71"/>
       <c r="H55" s="71" t="b">
         <v>0</v>
@@ -4827,7 +4861,7 @@
       <c r="E63" t="s">
         <v>472</v>
       </c>
-      <c r="F63" s="80" t="s">
+      <c r="F63" s="79" t="s">
         <v>655</v>
       </c>
       <c r="G63" s="71" t="s">
@@ -4872,7 +4906,7 @@
       <c r="E66" s="15" t="s">
         <v>505</v>
       </c>
-      <c r="F66" s="80" t="s">
+      <c r="F66" s="79" t="s">
         <v>531</v>
       </c>
       <c r="G66" s="72">
@@ -4926,7 +4960,7 @@
       <c r="E69" s="15" t="s">
         <v>536</v>
       </c>
-      <c r="F69" s="80" t="s">
+      <c r="F69" s="79" t="s">
         <v>657</v>
       </c>
       <c r="G69" t="s">
@@ -4951,7 +4985,7 @@
       <c r="G71" s="32" t="s">
         <v>660</v>
       </c>
-      <c r="H71" s="83" t="s">
+      <c r="H71" s="82" t="s">
         <v>661</v>
       </c>
       <c r="I71" s="14"/>
@@ -4980,7 +5014,7 @@
       <c r="E72" s="15" t="s">
         <v>481</v>
       </c>
-      <c r="F72" s="80" t="s">
+      <c r="F72" s="79" t="s">
         <v>542</v>
       </c>
       <c r="G72" s="71" t="s">
@@ -5028,7 +5062,7 @@
       <c r="E75" s="15" t="s">
         <v>512</v>
       </c>
-      <c r="F75" s="80" t="s">
+      <c r="F75" s="79" t="s">
         <v>668</v>
       </c>
       <c r="G75" s="72" t="b">
@@ -5078,7 +5112,7 @@
       <c r="E78" s="15" t="s">
         <v>513</v>
       </c>
-      <c r="F78" s="84" t="s">
+      <c r="F78" s="83" t="s">
         <v>534</v>
       </c>
       <c r="G78" s="72" t="b">
@@ -5123,7 +5157,7 @@
       <c r="E81" s="15" t="s">
         <v>521</v>
       </c>
-      <c r="F81" s="80" t="s">
+      <c r="F81" s="79" t="s">
         <v>662</v>
       </c>
       <c r="G81" s="72" t="s">
@@ -5187,7 +5221,7 @@
       <c r="E86" s="15" t="s">
         <v>514</v>
       </c>
-      <c r="F86" s="80" t="s">
+      <c r="F86" s="79" t="s">
         <v>663</v>
       </c>
       <c r="G86" s="72" t="b">
@@ -5233,7 +5267,7 @@
       <c r="E89" s="15" t="s">
         <v>515</v>
       </c>
-      <c r="F89" s="80" t="s">
+      <c r="F89" s="79" t="s">
         <v>664</v>
       </c>
       <c r="G89" s="72" t="b">
@@ -5258,7 +5292,7 @@
       <c r="C91">
         <v>88</v>
       </c>
-      <c r="G91" s="85" t="s">
+      <c r="G91" s="84" t="s">
         <v>329</v>
       </c>
       <c r="N91" s="62" t="s">
@@ -5285,7 +5319,7 @@
       <c r="E92" s="15" t="s">
         <v>517</v>
       </c>
-      <c r="F92" s="84" t="s">
+      <c r="F92" s="83" t="s">
         <v>532</v>
       </c>
       <c r="G92" s="74">
@@ -5347,7 +5381,7 @@
       <c r="E96" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="F96" s="80" t="s">
+      <c r="F96" s="79" t="s">
         <v>670</v>
       </c>
       <c r="G96" s="74">
@@ -5396,7 +5430,7 @@
       <c r="G100" s="1" t="s">
         <v>632</v>
       </c>
-      <c r="H100" s="88" t="s">
+      <c r="H100" s="87" t="s">
         <v>674</v>
       </c>
       <c r="I100" s="78"/>
@@ -5417,7 +5451,7 @@
       <c r="E101" s="15" t="s">
         <v>475</v>
       </c>
-      <c r="F101" s="80" t="s">
+      <c r="F101" s="79" t="s">
         <v>673</v>
       </c>
       <c r="G101" s="72" t="b">
@@ -5455,23 +5489,23 @@
         <v>634</v>
       </c>
     </row>
-    <row r="104" spans="1:16" s="80" customFormat="1" ht="17" thickTop="1" thickBot="1">
-      <c r="A104" s="80" t="s">
+    <row r="104" spans="1:16" s="79" customFormat="1" ht="17" thickTop="1" thickBot="1">
+      <c r="A104" s="79" t="s">
         <v>480</v>
       </c>
-      <c r="B104" s="80">
+      <c r="B104" s="79">
         <v>224</v>
       </c>
       <c r="C104">
         <v>101</v>
       </c>
-      <c r="D104" s="80" t="b">
-        <v>1</v>
-      </c>
-      <c r="E104" s="82" t="s">
+      <c r="D104" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="E104" s="81" t="s">
         <v>522</v>
       </c>
-      <c r="F104" s="89" t="s">
+      <c r="F104" s="88" t="s">
         <v>675</v>
       </c>
       <c r="G104" s="71" t="s">
@@ -5526,7 +5560,7 @@
       <c r="E107" s="15" t="s">
         <v>476</v>
       </c>
-      <c r="F107" s="89" t="s">
+      <c r="F107" s="88" t="s">
         <v>676</v>
       </c>
       <c r="G107" s="72" t="b">
@@ -5571,7 +5605,7 @@
       <c r="E110" s="15" t="s">
         <v>523</v>
       </c>
-      <c r="F110" s="89" t="s">
+      <c r="F110" s="88" t="s">
         <v>683</v>
       </c>
       <c r="G110" s="71" t="s">
@@ -5626,7 +5660,7 @@
       <c r="E113" s="15" t="s">
         <v>479</v>
       </c>
-      <c r="F113" s="89" t="s">
+      <c r="F113" s="88" t="s">
         <v>680</v>
       </c>
       <c r="G113" s="72" t="b">
@@ -5671,7 +5705,7 @@
       <c r="E116" s="15" t="s">
         <v>524</v>
       </c>
-      <c r="F116" s="89" t="s">
+      <c r="F116" s="88" t="s">
         <v>681</v>
       </c>
       <c r="G116" s="71" t="s">
@@ -5742,7 +5776,7 @@
       <c r="E121" s="15" t="s">
         <v>516</v>
       </c>
-      <c r="F121" s="89" t="s">
+      <c r="F121" s="88" t="s">
         <v>686</v>
       </c>
       <c r="G121" s="72" t="b">
@@ -5768,7 +5802,7 @@
       <c r="C123">
         <v>120</v>
       </c>
-      <c r="G123" s="85" t="s">
+      <c r="G123" s="84" t="s">
         <v>192</v>
       </c>
     </row>
@@ -5788,7 +5822,7 @@
       <c r="E124" s="15" t="s">
         <v>537</v>
       </c>
-      <c r="F124" s="84" t="s">
+      <c r="F124" s="83" t="s">
         <v>539</v>
       </c>
       <c r="G124" s="70" t="s">
@@ -5810,7 +5844,7 @@
       <c r="C126">
         <v>123</v>
       </c>
-      <c r="G126" s="85" t="s">
+      <c r="G126" s="84" t="s">
         <v>665</v>
       </c>
       <c r="N126" s="76" t="s">
@@ -5835,7 +5869,7 @@
       <c r="E127" s="15" t="s">
         <v>538</v>
       </c>
-      <c r="F127" s="84" t="s">
+      <c r="F127" s="83" t="s">
         <v>540</v>
       </c>
       <c r="G127" s="70" t="s">
@@ -5887,7 +5921,7 @@
       <c r="E130" s="15" t="s">
         <v>520</v>
       </c>
-      <c r="F130" s="80" t="s">
+      <c r="F130" s="79" t="s">
         <v>280</v>
       </c>
       <c r="G130" t="s">

</xml_diff>

<commit_message>
added TODO for dataframe reporting improvements; cleaned setup comment interference
Former-commit-id: 4d255634755e8f0696260c69b724a400e3d60517
</commit_message>
<xml_diff>
--- a/TestCampaign/ROVCleaver UniversalSetup.xlsx
+++ b/TestCampaign/ROVCleaver UniversalSetup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/TestInputFiles/TestCampaigns/BEK Test UniversalSetup/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/PythonProgs/ROVCleaver_on_Dropbox/TestCampaign/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F377F7A5-22DC-D640-B95E-80695A632667}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B8BF6F-DA16-D34F-AD6F-E01FA903827B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="24440" windowHeight="11500" activeTab="1" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="24440" windowHeight="11500" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="39" r:id="rId1"/>
@@ -3606,12 +3606,12 @@
   <dimension ref="A1:AD191"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1" outlineLevel="3"/>
-    <col min="2" max="3" width="8.1640625" customWidth="1" outlineLevel="3"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1" outlineLevel="3"/>
-    <col min="5" max="5" width="45" customWidth="1" outlineLevel="3"/>
-    <col min="6" max="6" width="38.6640625" style="81" customWidth="1" outlineLevel="2"/>
-    <col min="7" max="7" width="59.1640625" customWidth="1"/>
+    <col min="1" max="1" width="10" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="2" max="3" width="8.1640625" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="4" max="4" width="8.83203125" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="5" max="5" width="45" hidden="1" customWidth="1" outlineLevel="3"/>
+    <col min="6" max="6" width="38.6640625" style="81" hidden="1" customWidth="1" outlineLevel="2"/>
+    <col min="7" max="7" width="59.1640625" customWidth="1" collapsed="1"/>
     <col min="8" max="8" width="14.6640625" customWidth="1"/>
     <col min="9" max="9" width="12.33203125" customWidth="1"/>
     <col min="59" max="59" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -4226,6 +4226,9 @@
       <c r="G34" s="1" t="s">
         <v>601</v>
       </c>
+      <c r="H34" s="66" t="s">
+        <v>602</v>
+      </c>
     </row>
     <row r="35" spans="1:17" ht="17" thickTop="1" thickBot="1">
       <c r="A35" s="57" t="s">
@@ -4248,9 +4251,6 @@
       </c>
       <c r="G35" s="71" t="s">
         <v>54</v>
-      </c>
-      <c r="H35" s="66" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="36" spans="1:17" ht="16" thickTop="1">

</xml_diff>